<commit_message>
docs: complete analysis of oferta extraction and normalization results
Oferta 1:
- 1510 articles extracted (1267 referință + 243 supplement)
- 191 EXTRA: 136 breviar materials + 47 new articles + 8 from other devize (LEGITIMATE)
- 115 LIPSĂ: 65 absent from PDF + 50 match issues (ACCEPTABLE, no parser errors)
- Extraction quality: EXCELLENT (0 parser errors)

Oferta 2:
- 428 articles (incomplete - checkpoint was corrupted)
- Requires LLM re-classification to extract remaining 520 articles from PDFs
- API key needed

Oferta 3:
- 210 articles (incomplete - document has only ~17% of articles)
- Classification correct but document itself incomplete from contractor
- Not an extraction issue, but document design issue

All fixes applied:
- Deviz code normalization (U→0)
- Article code normalization (#)
- Result: 120 false EXTRA articles eliminated
</commit_message>
<xml_diff>
--- a/output_AO/Raport_Oferta_1.xlsx
+++ b/output_AO/Raport_Oferta_1.xlsx
@@ -890,8 +890,8 @@
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>$6753  ora  480.0
-Automacara cu brat cu zabrele 10- 14,9tf</t>
+          <t>$6752  ora  40.0
+Automacara 6- 9,9tf cu brat cu zabrele</t>
         </is>
       </c>
       <c r="D21" s="9" t="inlineStr">
@@ -932,8 +932,8 @@
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>CA01]1  mc  18.0
-Turnarea betonului simplu marca ... 1) in straturi de 5?20 cm, pentru egalizari, la constructii edilitare (apeducte, canale, anexe, etc.) material: manopera: utilaj: transport:</t>
+          <t>IZD03D1  tona  12.0
+Vopsire cu vops miniu cu aparat aer compr 1 str peconf si ctii metal exec din prof gros 8-12 MM material: manopera: utilaj: transport:</t>
         </is>
       </c>
       <c r="D23" s="9" t="inlineStr">
@@ -953,8 +953,8 @@
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
-          <t>IZD03D1  tona  12.0
-Vopsire cu vops miniu cu aparat aer compr 1 str peconf si ctii metal exec din prof gros 8-12 MM material: manopera: utilaj: transport:</t>
+          <t>IZD04D1  tona  12.0
+Vopsire cu aparat aer compr vopsea ulei pe conf siconstr met profile 8-12MM 2straturi material: manopera: utilaj: transport:</t>
         </is>
       </c>
       <c r="D24" s="9" t="inlineStr">
@@ -974,8 +974,8 @@
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>$6752  ora  40.0
-Automacara 6- 9,9tf cu brat cu zabrele</t>
+          <t>CA01]1  mc  18.0
+Turnarea betonului simplu marca ... 1) in straturi de 5?20 cm, pentru egalizari, la constructii edilitare (apeducte, canale, anexe, etc.) material: manopera: utilaj: transport:</t>
         </is>
       </c>
       <c r="D25" s="9" t="inlineStr">
@@ -995,8 +995,8 @@
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
-          <t>$226108    0.0
-STRUCTURA DE REZISTENTA CUPOLA TEREN TENIS e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
+          <t>$6753  ora  480.0
+Automacara cu brat cu zabrele 10- 14,9tf</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
@@ -1016,8 +1016,8 @@
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>IZD04D1  tona  12.0
-Vopsire cu aparat aer compr vopsea ulei pe conf siconstr met profile 8-12MM 2straturi material: manopera: utilaj: transport:</t>
+          <t>$226108    0.0
+STRUCTURA DE REZISTENTA CUPOLA TEREN TENIS e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr">
@@ -1268,8 +1268,8 @@
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
-          <t>$3336  ora  64.0
-Pompa hidraulica de beton cu 100M conducta,pina la 40 MC/H</t>
+          <t>$226208    0.0
+STRUCTURA DE REZISTENTA (vestiar, grupuri sanitare) e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
         </is>
       </c>
       <c r="D39" s="9" t="inlineStr">
@@ -1289,8 +1289,8 @@
       </c>
       <c r="C40" s="8" t="inlineStr">
         <is>
-          <t>$226208    0.0
-STRUCTURA DE REZISTENTA (vestiar, grupuri sanitare) e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
+          <t>$6752  ora  64.0
+Automacara 6- 9,9tf cu brat cu zabrele</t>
         </is>
       </c>
       <c r="D40" s="9" t="inlineStr">
@@ -1310,8 +1310,8 @@
       </c>
       <c r="C41" s="8" t="inlineStr">
         <is>
-          <t>$6311528  kg  46.8
-Scoaba otel pentru constructii din lemn, latime= 65-90MM, L.200-300 MM</t>
+          <t>$3336  ora  64.0
+Pompa hidraulica de beton cu 100M conducta,pina la 40 MC/H</t>
         </is>
       </c>
       <c r="D41" s="9" t="inlineStr">
@@ -1331,8 +1331,8 @@
       </c>
       <c r="C42" s="8" t="inlineStr">
         <is>
-          <t>$6752  ora  64.0
-Automacara 6- 9,9tf cu brat cu zabrele</t>
+          <t>$6311528  kg  46.8
+Scoaba otel pentru constructii din lemn, latime= 65-90MM, L.200-300 MM</t>
         </is>
       </c>
       <c r="D42" s="9" t="inlineStr">
@@ -1734,8 +1734,8 @@
       </c>
       <c r="C61" s="8" t="inlineStr">
         <is>
-          <t>CE23A1  mp  1256.0
-Plasa de siguranta, refolosibila, la executarea invelitorii constructiilor</t>
+          <t>RPCE29A  mp  1256.0
+Prelata pentru protejarea terasei pe timp ploios pe durata refacerii</t>
         </is>
       </c>
       <c r="D61" s="9" t="inlineStr">
@@ -1755,8 +1755,8 @@
       </c>
       <c r="C62" s="8" t="inlineStr">
         <is>
-          <t>$6306431  mp  7.0
-USI DIN PVC</t>
+          <t>$7800859  kg  39.5
+Vopsea lavabila acrilica</t>
         </is>
       </c>
       <c r="D62" s="9" t="inlineStr">
@@ -1776,8 +1776,8 @@
       </c>
       <c r="C63" s="8" t="inlineStr">
         <is>
-          <t>$1303  ora  2160.0
-Schela met tubext.S640mp G=11-13,5 3sch.lei/mp</t>
+          <t>$3999988  mp  1256.0
+PRELATA SPECIALA ANTIVANT, REZISTENT LA FOC, LA UMIDITATE SI MUCEGAI</t>
         </is>
       </c>
       <c r="D63" s="9" t="inlineStr">
@@ -1797,8 +1797,7 @@
       </c>
       <c r="C64" s="8" t="inlineStr">
         <is>
-          <t>$16509  mp  230.0
-VOPSITORIE DECORATIVA material: manopera: utilaj: transport:</t>
+          <t>S7064  kg  60.0</t>
         </is>
       </c>
       <c r="D64" s="9" t="inlineStr">
@@ -1818,8 +1817,8 @@
       </c>
       <c r="C65" s="8" t="inlineStr">
         <is>
-          <t>$7800857  kg  7.9
-Amorsa pt. vopsea lavabila</t>
+          <t>TRB05B23  tona  25.0
+Transportul materialelor prin purtat direct,materiale incomode peste 25 Kg distanta 30M</t>
         </is>
       </c>
       <c r="D65" s="9" t="inlineStr">
@@ -1839,8 +1838,8 @@
       </c>
       <c r="C66" s="8" t="inlineStr">
         <is>
-          <t>$2941123  mp  1256.0
-PLASA TEXTILA 2 MM PENTRU CUPOLE TEREN</t>
+          <t>$71100101  m  19.95
+@JGHEAB TABLA VOPSITA ELECTROSTATIC DE 15 CM</t>
         </is>
       </c>
       <c r="D66" s="9" t="inlineStr">
@@ -1860,8 +1859,8 @@
       </c>
       <c r="C67" s="8" t="inlineStr">
         <is>
-          <t>$7800859  kg  39.5
-Vopsea lavabila acrilica</t>
+          <t>$4741  kg  736.0
+71</t>
         </is>
       </c>
       <c r="D67" s="9" t="inlineStr">
@@ -1881,7 +1880,8 @@
       </c>
       <c r="C68" s="8" t="inlineStr">
         <is>
-          <t>S7064  kg  60.0</t>
+          <t>$7800774  mp  188.76
+Folie anticondens</t>
         </is>
       </c>
       <c r="D68" s="9" t="inlineStr">
@@ -1901,8 +1901,8 @@
       </c>
       <c r="C69" s="8" t="inlineStr">
         <is>
-          <t>$22041951  m  9.0
-GLAF EXT TABLA VOPSITA 25 CM, CU PICURATOR SI ACCESORII PE MONTAJ Deviz "226218" - Formular F3 Formular generat cu programul Devize (www.eDevize.ro) Pagina 5 din 8</t>
+          <t>$71100111  m  7.35
+@BURLAN DIN TABLA VOPSITA ELECTROSTATIC DE DN=15 CM</t>
         </is>
       </c>
       <c r="D69" s="9" t="inlineStr">
@@ -1922,8 +1922,8 @@
       </c>
       <c r="C70" s="8" t="inlineStr">
         <is>
-          <t>TRB05B23  tona  25.0
-Transportul materialelor prin purtat direct,materiale incomode peste 25 Kg distanta 30M</t>
+          <t>$7800857  kg  7.9
+Amorsa pt. vopsea lavabila</t>
         </is>
       </c>
       <c r="D70" s="9" t="inlineStr">
@@ -1943,8 +1943,8 @@
       </c>
       <c r="C71" s="8" t="inlineStr">
         <is>
-          <t>$71100101  m  19.95
-@JGHEAB TABLA VOPSITA ELECTROSTATIC DE 15 CM</t>
+          <t>$22041951  m  9.0
+GLAF EXT TABLA VOPSITA 25 CM, CU PICURATOR SI ACCESORII PE MONTAJ Deviz "226218" - Formular F3 Formular generat cu programul Devize (www.eDevize.ro) Pagina 5 din 8</t>
         </is>
       </c>
       <c r="D71" s="9" t="inlineStr">
@@ -1964,8 +1964,8 @@
       </c>
       <c r="C72" s="8" t="inlineStr">
         <is>
-          <t>$7800774  mp  188.76
-Folie anticondens</t>
+          <t>$226218    0.0
+ARHITECTURA teren tenis si grupuri sanitare eDevize e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
         </is>
       </c>
       <c r="D72" s="9" t="inlineStr">
@@ -1985,8 +1985,8 @@
       </c>
       <c r="C73" s="8" t="inlineStr">
         <is>
-          <t>CK25A  mp  7.0
-Usi profiluri mase plastice, 1 canat, supraf toc &lt;= 7 mp,inclusiv armaturi si accesorii,montate in zid de orice fel la constructii cu H &lt;= 35 M</t>
+          <t>$6306493  mp  34.0
+USA PVC</t>
         </is>
       </c>
       <c r="D73" s="9" t="inlineStr">
@@ -2006,8 +2006,8 @@
       </c>
       <c r="C74" s="8" t="inlineStr">
         <is>
-          <t>PF04A1ASIM  mp  79.0
-STRAT AMORSAJ APLICAT CU PERIA DIN BITUM TAIAT CU WHITE SPIRIT RAFINAT</t>
+          <t>$16509  mp  230.0
+VOPSITORIE DECORATIVA material: manopera: utilaj: transport:</t>
         </is>
       </c>
       <c r="D74" s="9" t="inlineStr">
@@ -2027,8 +2027,8 @@
       </c>
       <c r="C75" s="8" t="inlineStr">
         <is>
-          <t>$4741  kg  736.0
-71</t>
+          <t>$2941123  mp  1256.0
+PLASA TEXTILA 2 MM PENTRU CUPOLE TEREN</t>
         </is>
       </c>
       <c r="D75" s="9" t="inlineStr">
@@ -2048,8 +2048,8 @@
       </c>
       <c r="C76" s="8" t="inlineStr">
         <is>
-          <t>$16508  mp  230.0
-SISTEM TERMOIZ. CU VATA MINERALA B material: manopera: utilaj: transport:</t>
+          <t>PF04A1ASIM  mp  79.0
+STRAT AMORSAJ APLICAT CU PERIA DIN BITUM TAIAT CU WHITE SPIRIT RAFINAT</t>
         </is>
       </c>
       <c r="D76" s="9" t="inlineStr">
@@ -2069,8 +2069,8 @@
       </c>
       <c r="C77" s="8" t="inlineStr">
         <is>
-          <t>$71100111  m  7.35
-@BURLAN DIN TABLA VOPSITA ELECTROSTATIC DE DN=15 CM</t>
+          <t>$1303  ora  2160.0
+Schela met tubext.S640mp G=11-13,5 3sch.lei/mp</t>
         </is>
       </c>
       <c r="D77" s="9" t="inlineStr">
@@ -2090,8 +2090,8 @@
       </c>
       <c r="C78" s="8" t="inlineStr">
         <is>
-          <t>$6306493  mp  34.0
-USA PVC</t>
+          <t>$32742701  kg  15.0
+Adeziv granit</t>
         </is>
       </c>
       <c r="D78" s="9" t="inlineStr">
@@ -2111,8 +2111,8 @@
       </c>
       <c r="C79" s="8" t="inlineStr">
         <is>
-          <t>$3999988  mp  1256.0
-PRELATA SPECIALA ANTIVANT, REZISTENT LA FOC, LA UMIDITATE SI MUCEGAI</t>
+          <t>CE23A1  mp  1256.0
+Plasa de siguranta, refolosibila, la executarea invelitorii constructiilor</t>
         </is>
       </c>
       <c r="D79" s="9" t="inlineStr">
@@ -2132,8 +2132,8 @@
       </c>
       <c r="C80" s="8" t="inlineStr">
         <is>
-          <t>$226218    0.0
-ARHITECTURA teren tenis si grupuri sanitare eDevize e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
+          <t>$6306431  mp  7.0
+USI DIN PVC</t>
         </is>
       </c>
       <c r="D80" s="9" t="inlineStr">
@@ -2153,8 +2153,8 @@
       </c>
       <c r="C81" s="8" t="inlineStr">
         <is>
-          <t>RPCE29A  mp  1256.0
-Prelata pentru protejarea terasei pe timp ploios pe durata refacerii</t>
+          <t>$16508  mp  230.0
+SISTEM TERMOIZ. CU VATA MINERALA B material: manopera: utilaj: transport:</t>
         </is>
       </c>
       <c r="D81" s="9" t="inlineStr">
@@ -2174,8 +2174,8 @@
       </c>
       <c r="C82" s="8" t="inlineStr">
         <is>
-          <t>$32742701  kg  15.0
-Adeziv granit</t>
+          <t>CK25A  mp  7.0
+Usi profiluri mase plastice, 1 canat, supraf toc &lt;= 7 mp,inclusiv armaturi si accesorii,montate in zid de orice fel la constructii cu H &lt;= 35 M</t>
         </is>
       </c>
       <c r="D82" s="9" t="inlineStr">
@@ -2719,8 +2719,8 @@
       </c>
       <c r="C107" s="8" t="inlineStr">
         <is>
-          <t>$2222219  buc  4.0
-CADITE DUS</t>
+          <t>$30001  ora  0.5
+APARAT DE SUDURA COPRAX 2204/ /50Hz/700w</t>
         </is>
       </c>
       <c r="D107" s="9" t="inlineStr">
@@ -2740,8 +2740,8 @@
       </c>
       <c r="C108" s="8" t="inlineStr">
         <is>
-          <t>$05021  buc  9.0
-MONTAT LAVOAR GRUP SANITAR material: manopera: utilaj: transport:</t>
+          <t>$327101  m  30.6
+TEAVA PN20 PPR VERDE DN32</t>
         </is>
       </c>
       <c r="D108" s="9" t="inlineStr">
@@ -2761,8 +2761,7 @@
       </c>
       <c r="C109" s="8" t="inlineStr">
         <is>
-          <t>$05024  buc  4.0
-MONTAT DUS GRUP SANITAR material: manopera: utilaj: transport:</t>
+          <t>S9610  buc  1.0</t>
         </is>
       </c>
       <c r="D109" s="9" t="inlineStr">
@@ -2782,7 +2781,8 @@
       </c>
       <c r="C110" s="8" t="inlineStr">
         <is>
-          <t>S9610  buc  1.0</t>
+          <t>$05027  buc  1.0
+MONTAT WC PERSOANE CU DIZABILITATI material: manopera: utilaj: transport:</t>
         </is>
       </c>
       <c r="D110" s="9" t="inlineStr">
@@ -2802,8 +2802,8 @@
       </c>
       <c r="C111" s="8" t="inlineStr">
         <is>
-          <t>$30001  ora  0.5
-APARAT DE SUDURA COPRAX 2204/ /50Hz/700w</t>
+          <t>$24384071  buc  9.0
+Lavoar portelan</t>
         </is>
       </c>
       <c r="D111" s="9" t="inlineStr">
@@ -2823,8 +2823,8 @@
       </c>
       <c r="C112" s="8" t="inlineStr">
         <is>
-          <t>$3210241  buc  4.0
-Teu egal PPR 32</t>
+          <t>$05024  buc  4.0
+MONTAT DUS GRUP SANITAR material: manopera: utilaj: transport:</t>
         </is>
       </c>
       <c r="D112" s="9" t="inlineStr">
@@ -2844,8 +2844,8 @@
       </c>
       <c r="C113" s="8" t="inlineStr">
         <is>
-          <t>$05027  buc  1.0
-MONTAT WC PERSOANE CU DIZABILITATI material: manopera: utilaj: transport:</t>
+          <t>$05021  buc  9.0
+MONTAT LAVOAR GRUP SANITAR material: manopera: utilaj: transport:</t>
         </is>
       </c>
       <c r="D113" s="9" t="inlineStr">
@@ -2865,8 +2865,8 @@
       </c>
       <c r="C114" s="8" t="inlineStr">
         <is>
-          <t>$05028  buc  1.0
-MONTAT LAVOAR PERSOANE CU DIZABILITATI material: manopera: utilaj: transport:</t>
+          <t>$3210241  buc  4.0
+Teu egal PPR 32</t>
         </is>
       </c>
       <c r="D114" s="9" t="inlineStr">
@@ -2886,8 +2886,8 @@
       </c>
       <c r="C115" s="8" t="inlineStr">
         <is>
-          <t>$24384071  buc  9.0
-Lavoar portelan</t>
+          <t>$2222219  buc  4.0
+CADITE DUS</t>
         </is>
       </c>
       <c r="D115" s="9" t="inlineStr">
@@ -2907,8 +2907,8 @@
       </c>
       <c r="C116" s="8" t="inlineStr">
         <is>
-          <t>$05022  buc  4.0
-MONTAT WC GRUP SANITAR material: manopera: utilaj: transport:</t>
+          <t>$3211097  buc  4.0
+REDUCTIE PPR 40-32</t>
         </is>
       </c>
       <c r="D116" s="9" t="inlineStr">
@@ -2928,8 +2928,8 @@
       </c>
       <c r="C117" s="8" t="inlineStr">
         <is>
-          <t>$327101  m  30.6
-TEAVA PN20 PPR VERDE DN32</t>
+          <t>$05028  buc  1.0
+MONTAT LAVOAR PERSOANE CU DIZABILITATI material: manopera: utilaj: transport:</t>
         </is>
       </c>
       <c r="D117" s="9" t="inlineStr">
@@ -2949,8 +2949,8 @@
       </c>
       <c r="C118" s="8" t="inlineStr">
         <is>
-          <t>$3211097  buc  4.0
-REDUCTIE PPR 40-32</t>
+          <t>$05022  buc  4.0
+MONTAT WC GRUP SANITAR material: manopera: utilaj: transport:</t>
         </is>
       </c>
       <c r="D118" s="9" t="inlineStr">
@@ -3441,8 +3441,8 @@
       </c>
       <c r="C142" s="8" t="inlineStr">
         <is>
-          <t>$63100311  kg  46000.0
-CONFECTII METALICE APARENTA</t>
+          <t>$63022421  kg  21800.0
+Stilp din otel</t>
         </is>
       </c>
       <c r="D142" s="9" t="inlineStr">
@@ -3462,8 +3462,8 @@
       </c>
       <c r="C143" s="8" t="inlineStr">
         <is>
-          <t>$63047211  kg  16800.0
-Pana otel Deviz "226308" - Formular F3 Formular generat cu programul @Devize (www.eDevize.ro) Pagina 4 din 6</t>
+          <t>IZD03D1  tona  96.8
+Vopsire cu vops miniu cu aparat aer compr 1 str peconf si ctii metal exec din prof gros 8-12 MM</t>
         </is>
       </c>
       <c r="D143" s="9" t="inlineStr">
@@ -3483,8 +3483,8 @@
       </c>
       <c r="C144" s="8" t="inlineStr">
         <is>
-          <t>$32745862  kg  4466.0
-OTEL BETON BST500 10-16 mm</t>
+          <t>$63000241  kg  12200.0
+Grinda otel</t>
         </is>
       </c>
       <c r="D144" s="9" t="inlineStr">
@@ -3504,8 +3504,8 @@
       </c>
       <c r="C145" s="8" t="inlineStr">
         <is>
-          <t>$226308    0.0
-STRUCTURA DE REZISTENTA- (gradene 2 BUC) e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
+          <t>$32745862  kg  4466.0
+OTEL BETON BST500 10-16 mm</t>
         </is>
       </c>
       <c r="D145" s="9" t="inlineStr">
@@ -3525,8 +3525,8 @@
       </c>
       <c r="C146" s="8" t="inlineStr">
         <is>
-          <t>$63022421  kg  21800.0
-Stilp din otel</t>
+          <t>IZD04D1  tona  96.8
+Vopsire cu aparat aer compr vopsea ulei pe conf siconstr met profile 8-12MM 2straturi</t>
         </is>
       </c>
       <c r="D146" s="9" t="inlineStr">
@@ -3546,8 +3546,8 @@
       </c>
       <c r="C147" s="8" t="inlineStr">
         <is>
-          <t>IZD04D1  tona  96.8
-Vopsire cu aparat aer compr vopsea ulei pe conf siconstr met profile 8-12MM 2straturi</t>
+          <t>$63047211  kg  16800.0
+Pana otel Deviz "226308" - Formular F3 Formular generat cu programul @Devize (www.eDevize.ro) Pagina 4 din 6</t>
         </is>
       </c>
       <c r="D147" s="9" t="inlineStr">
@@ -3567,8 +3567,8 @@
       </c>
       <c r="C148" s="8" t="inlineStr">
         <is>
-          <t>$3336  ora  80.0
-Pompa hidraulica de beton cu 100M conducta, pina la 40 MC/H</t>
+          <t>$63100311  kg  46000.0
+CONFECTII METALICE APARENTA</t>
         </is>
       </c>
       <c r="D148" s="9" t="inlineStr">
@@ -3588,8 +3588,8 @@
       </c>
       <c r="C149" s="8" t="inlineStr">
         <is>
-          <t>$63000241  kg  12200.0
-Grinda otel</t>
+          <t>$226308    0.0
+STRUCTURA DE REZISTENTA- (gradene 2 BUC) e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
         </is>
       </c>
       <c r="D149" s="9" t="inlineStr">
@@ -3609,8 +3609,8 @@
       </c>
       <c r="C150" s="8" t="inlineStr">
         <is>
-          <t>IZD03D1  tona  96.8
-Vopsire cu vops miniu cu aparat aer compr 1 str peconf si ctii metal exec din prof gros 8-12 MM</t>
+          <t>$6752  ora  480.0
+Automacara 6- 9,9tf cu brat cu zabrele</t>
         </is>
       </c>
       <c r="D150" s="9" t="inlineStr">
@@ -3630,8 +3630,8 @@
       </c>
       <c r="C151" s="8" t="inlineStr">
         <is>
-          <t>$6752  ora  480.0
-Automacara 6- 9,9tf cu brat cu zabrele</t>
+          <t>$3336  ora  80.0
+Pompa hidraulica de beton cu 100M conducta, pina la 40 MC/H</t>
         </is>
       </c>
       <c r="D151" s="9" t="inlineStr">
@@ -3950,8 +3950,8 @@
       </c>
       <c r="C167" s="8" t="inlineStr">
         <is>
-          <t>$26012091  mp  9244.0
-Membrana hidroizolatoare bituminoasa antiacida</t>
+          <t>$20010472  mc  2522.0
+Pamant vegetal Deviz "226338" - Formular F3 Formular generat cu programul Devize (www.eDevize.ro) Pagina 1 din 3</t>
         </is>
       </c>
       <c r="D167" s="9" t="inlineStr">
@@ -3992,8 +3992,8 @@
       </c>
       <c r="C169" s="8" t="inlineStr">
         <is>
-          <t>IZD04D1  tona  12.85
-Vopsire cu aparat aer compr vopsea ulei pe conf siconstr met profile 8-12MM 2straturi</t>
+          <t>$26012091  mp  9244.0
+Membrana hidroizolatoare bituminoasa antiacida</t>
         </is>
       </c>
       <c r="D169" s="9" t="inlineStr">
@@ -4013,8 +4013,8 @@
       </c>
       <c r="C170" s="8" t="inlineStr">
         <is>
-          <t>$20010472  mc  2522.0
-Pamant vegetal Deviz "226338" - Formular F3 Formular generat cu programul Devize (www.eDevize.ro) Pagina 1 din 3</t>
+          <t>IZD03D1  tona  12.85
+Vopsire cu vops miniu cu aparat aer compr 1 str peconf si ctii metal exec din prof gros 8-12 MM</t>
         </is>
       </c>
       <c r="D170" s="9" t="inlineStr">
@@ -4034,8 +4034,8 @@
       </c>
       <c r="C171" s="8" t="inlineStr">
         <is>
-          <t>$226318    0.0
-ÎMPREJMUIRE TEREN FOTBAL -380 ML e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
+          <t>IZD04D1  tona  12.85
+Vopsire cu aparat aer compr vopsea ulei pe conf siconstr met profile 8-12MM 2straturi</t>
         </is>
       </c>
       <c r="D171" s="9" t="inlineStr">
@@ -4055,8 +4055,8 @@
       </c>
       <c r="C172" s="8" t="inlineStr">
         <is>
-          <t>IZD03D1  tona  12.85
-Vopsire cu vops miniu cu aparat aer compr 1 str peconf si ctii metal exec din prof gros 8-12 MM</t>
+          <t>$226318    0.0
+ÎMPREJMUIRE TEREN FOTBAL -380 ML e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
         </is>
       </c>
       <c r="D172" s="9" t="inlineStr">
@@ -4339,8 +4339,8 @@
       </c>
       <c r="C186" s="8" t="inlineStr">
         <is>
-          <t>TRA01A20P  tona  1132.4
-Transportul rutier al pamantului sau molozului cu autobasculanta dist .= 20 km material: manopera: utilaj: transport:</t>
+          <t>$22000561  mc  100.0
+Pietris concasat sort 4-8 mm</t>
         </is>
       </c>
       <c r="D186" s="9" t="inlineStr">
@@ -4360,8 +4360,8 @@
       </c>
       <c r="C187" s="8" t="inlineStr">
         <is>
-          <t>$226358    0.0
-ALEI PIETONALE SI CAROSABILE e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
+          <t>TRA01A20P  tona  1132.4
+Transportul rutier al pamantului sau molozului cu autobasculanta dist .= 20 km material: manopera: utilaj: transport:</t>
         </is>
       </c>
       <c r="D187" s="9" t="inlineStr">
@@ -4381,8 +4381,8 @@
       </c>
       <c r="C188" s="8" t="inlineStr">
         <is>
-          <t>$22000561  mc  100.0
-Pietris concasat sort 4-8 mm</t>
+          <t>$22100100  mp  2000.0
+PROFIL FAGURE ECOLOGIC</t>
         </is>
       </c>
       <c r="D188" s="9" t="inlineStr">
@@ -4402,8 +4402,8 @@
       </c>
       <c r="C189" s="8" t="inlineStr">
         <is>
-          <t>$22100100  mp  2000.0
-PROFIL FAGURE ECOLOGIC</t>
+          <t>$226358    0.0
+ALEI PIETONALE SI CAROSABILE e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
         </is>
       </c>
       <c r="D189" s="9" t="inlineStr">
@@ -4738,8 +4738,8 @@
       </c>
       <c r="C205" s="8" t="inlineStr">
         <is>
-          <t>CB13I1  mp  300.0
-Cofraje pentru beton armat in placi, grinzi si stilpi din panouri refolosibile, cu placaj' de 15 mm grosime la constructii avand inaltimea pana la 20 m inclusiv, la placi si grinzi; material: manopera: utilaj: transport:</t>
+          <t>IZD04D1  tona  0.95
+Vopsire cu aparat aer compr vopsea ulei pe conf siconstr met profile 8-12MM 2straturi material: manopera: utilaj: transport:</t>
         </is>
       </c>
       <c r="D205" s="9" t="inlineStr">
@@ -4759,8 +4759,8 @@
       </c>
       <c r="C206" s="8" t="inlineStr">
         <is>
-          <t>IZD03D1  tona  0.95
-Vopsire cu vops miniu cu aparat aer compr 1 str peconf si ctii metal exec din prof gros 8-12 MM material: manopera: utilaj: transport:</t>
+          <t>$63100311  kg  950.0
+CONFECTII METALICE APARENTA</t>
         </is>
       </c>
       <c r="D206" s="9" t="inlineStr">
@@ -4780,8 +4780,8 @@
       </c>
       <c r="C207" s="8" t="inlineStr">
         <is>
-          <t>$63100311  kg  950.0
-CONFECTII METALICE APARENTA</t>
+          <t>$32745863  kg  5582.5
+OTEL BETON BST500 10-16</t>
         </is>
       </c>
       <c r="D207" s="9" t="inlineStr">
@@ -4801,8 +4801,8 @@
       </c>
       <c r="C208" s="8" t="inlineStr">
         <is>
-          <t>$226408    0.0
-STRUCTURA DE REZISTENTA {vestiare, sala fitness) e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
+          <t>S7064  kg  45.0
+Deviz "226408" - Formular F3 Formular generat cu programul @Devize (www.eDevize.ro) Pagina 3 din 7</t>
         </is>
       </c>
       <c r="D208" s="9" t="inlineStr">
@@ -4822,8 +4822,8 @@
       </c>
       <c r="C209" s="8" t="inlineStr">
         <is>
-          <t>IZD04D1  tona  0.95
-Vopsire cu aparat aer compr vopsea ulei pe conf siconstr met profile 8-12MM 2straturi material: manopera: utilaj: transport:</t>
+          <t>$32745843  kg  588.7
+OTEL BETON BST500 6-8</t>
         </is>
       </c>
       <c r="D209" s="9" t="inlineStr">
@@ -4843,8 +4843,8 @@
       </c>
       <c r="C210" s="8" t="inlineStr">
         <is>
-          <t>$32745863  kg  5582.5
-OTEL BETON BST500 10-16</t>
+          <t>CB13I1  mp  300.0
+Cofraje pentru beton armat in placi, grinzi si stilpi din panouri refolosibile, cu placaj' de 15 mm grosime la constructii avand inaltimea pana la 20 m inclusiv, la placi si grinzi; material: manopera: utilaj: transport:</t>
         </is>
       </c>
       <c r="D210" s="9" t="inlineStr">
@@ -4864,8 +4864,8 @@
       </c>
       <c r="C211" s="8" t="inlineStr">
         <is>
-          <t>$32745843  kg  588.7
-OTEL BETON BST500 6-8</t>
+          <t>$226408    0.0
+STRUCTURA DE REZISTENTA {vestiare, sala fitness) e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
         </is>
       </c>
       <c r="D211" s="9" t="inlineStr">
@@ -4885,8 +4885,8 @@
       </c>
       <c r="C212" s="8" t="inlineStr">
         <is>
-          <t>S7064  kg  45.0
-Deviz "226408" - Formular F3 Formular generat cu programul @Devize (www.eDevize.ro) Pagina 3 din 7</t>
+          <t>IZD03D1  tona  0.95
+Vopsire cu vops miniu cu aparat aer compr 1 str peconf si ctii metal exec din prof gros 8-12 MM material: manopera: utilaj: transport:</t>
         </is>
       </c>
       <c r="D212" s="9" t="inlineStr">
@@ -5292,8 +5292,8 @@
       </c>
       <c r="C231" s="8" t="inlineStr">
         <is>
-          <t>$6306493  mp  47.0
-USA PVC Deviz "226418" - Formular F3 Formular generat cu programul @Devize (www.eDevize.ro) Pagina 5 din 8</t>
+          <t>$7800774  mp  225.0
+Folie anticondens</t>
         </is>
       </c>
       <c r="D231" s="9" t="inlineStr">
@@ -5313,8 +5313,8 @@
       </c>
       <c r="C232" s="8" t="inlineStr">
         <is>
-          <t>$226418    0.0
-ARHITECTURA VESTIARE FOTBALIST SI SALA FITNESS e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
+          <t>PF04A1ASIM  mp  241.0
+STRAT AMORSAJ APLICAT CU PERIA DIN BITUM TAIAT CU WHITE SPIRIT RAFINAT</t>
         </is>
       </c>
       <c r="D232" s="9" t="inlineStr">
@@ -5334,7 +5334,8 @@
       </c>
       <c r="C233" s="8" t="inlineStr">
         <is>
-          <t>S7064  kg  90.0</t>
+          <t>$22041951  m  21.0
+GLAF EXT TABLA VOPSITA 25 CM, CU PICURATOR SI ACCESORII PE MONTAJ</t>
         </is>
       </c>
       <c r="D233" s="9" t="inlineStr">
@@ -5354,8 +5355,8 @@
       </c>
       <c r="C234" s="8" t="inlineStr">
         <is>
-          <t>$22041951  m  21.0
-GLAF EXT TABLA VOPSITA 25 CM, CU PICURATOR SI ACCESORII PE MONTAJ</t>
+          <t>$226418    0.0
+ARHITECTURA VESTIARE FOTBALIST SI SALA FITNESS e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
         </is>
       </c>
       <c r="D234" s="9" t="inlineStr">
@@ -5375,8 +5376,8 @@
       </c>
       <c r="C235" s="8" t="inlineStr">
         <is>
-          <t>RPCR21A1  mp  591.0
-Vopsitorii interioare cu vopsea lavabila la pereti si tavane cu vopsea lavabila,pe glet de ipsos material: manopera: utilaj: transport:</t>
+          <t>$6306493  mp  47.0
+USA PVC Deviz "226418" - Formular F3 Formular generat cu programul @Devize (www.eDevize.ro) Pagina 5 din 8</t>
         </is>
       </c>
       <c r="D235" s="9" t="inlineStr">
@@ -5396,8 +5397,8 @@
       </c>
       <c r="C236" s="8" t="inlineStr">
         <is>
-          <t>$16509  mp  416.0
-VOPSITORIE DECORATIVA material: manopera: utilaj: transport:</t>
+          <t>RPCR21A1  mp  591.0
+Vopsitorii interioare cu vopsea lavabila la pereti si tavane cu vopsea lavabila,pe glet de ipsos material: manopera: utilaj: transport:</t>
         </is>
       </c>
       <c r="D236" s="9" t="inlineStr">
@@ -5417,8 +5418,8 @@
       </c>
       <c r="C237" s="8" t="inlineStr">
         <is>
-          <t>$7800859  kg  120.5
-Vopsea lavabila acrilica</t>
+          <t>$32742701  kg  8.5
+Adeziv granit</t>
         </is>
       </c>
       <c r="D237" s="9" t="inlineStr">
@@ -5438,8 +5439,8 @@
       </c>
       <c r="C238" s="8" t="inlineStr">
         <is>
-          <t>$7800774  mp  225.0
-Folie anticondens</t>
+          <t>$7800859  kg  120.5
+Vopsea lavabila acrilica</t>
         </is>
       </c>
       <c r="D238" s="9" t="inlineStr">
@@ -5480,8 +5481,8 @@
       </c>
       <c r="C240" s="8" t="inlineStr">
         <is>
-          <t>$71100111  m  14.7
-@BURLAN DIN TABLA VOPSITA ELECTROSTATIC DE DN=15 CM</t>
+          <t>$71100101  m  14.7
+@JGHEAB TABLA VOPSITA ELECTROSTATIC DE 15 CM</t>
         </is>
       </c>
       <c r="D240" s="9" t="inlineStr">
@@ -5501,8 +5502,8 @@
       </c>
       <c r="C241" s="8" t="inlineStr">
         <is>
-          <t>$71100101  m  14.7
-@JGHEAB TABLA VOPSITA ELECTROSTATIC DE 15 CM</t>
+          <t>$16509  mp  416.0
+VOPSITORIE DECORATIVA material: manopera: utilaj: transport:</t>
         </is>
       </c>
       <c r="D241" s="9" t="inlineStr">
@@ -5522,8 +5523,8 @@
       </c>
       <c r="C242" s="8" t="inlineStr">
         <is>
-          <t>$32742701  kg  8.5
-Adeziv granit</t>
+          <t>$4741  kg  1331.2
+71</t>
         </is>
       </c>
       <c r="D242" s="9" t="inlineStr">
@@ -5543,8 +5544,8 @@
       </c>
       <c r="C243" s="8" t="inlineStr">
         <is>
-          <t>PF04A1ASIM  mp  241.0
-STRAT AMORSAJ APLICAT CU PERIA DIN BITUM TAIAT CU WHITE SPIRIT RAFINAT</t>
+          <t>$71100111  m  14.7
+@BURLAN DIN TABLA VOPSITA ELECTROSTATIC DE DN=15 CM</t>
         </is>
       </c>
       <c r="D243" s="9" t="inlineStr">
@@ -5564,8 +5565,7 @@
       </c>
       <c r="C244" s="8" t="inlineStr">
         <is>
-          <t>$4741  kg  1331.2
-71</t>
+          <t>S7064  kg  90.0</t>
         </is>
       </c>
       <c r="D244" s="9" t="inlineStr">
@@ -5877,8 +5877,8 @@
       </c>
       <c r="C259" s="8" t="inlineStr">
         <is>
-          <t>$226228    0.0
-INSTALATII SANITARE OB.2 e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
+          <t>$226428    0.0
+INSTALATII SANITARE OB 4 e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
         </is>
       </c>
       <c r="D259" s="9" t="inlineStr">
@@ -5898,8 +5898,7 @@
       </c>
       <c r="C260" s="8" t="inlineStr">
         <is>
-          <t>$32719871  buc  3.0
-ROBINET SFERA APA 1"1/4 GIACOMINI DN 32 R 250</t>
+          <t>N1080  buc  9.0</t>
         </is>
       </c>
       <c r="D260" s="9" t="inlineStr">
@@ -5919,7 +5918,8 @@
       </c>
       <c r="C261" s="8" t="inlineStr">
         <is>
-          <t>N1080  buc  9.0</t>
+          <t>$32719861  buc  3.0
+ROBINET SFERA APA 1"GIACOMINI DN 25 R</t>
         </is>
       </c>
       <c r="D261" s="9" t="inlineStr">
@@ -5939,8 +5939,8 @@
       </c>
       <c r="C262" s="8" t="inlineStr">
         <is>
-          <t>$2222219  buc  3.0
-CADITE DUS</t>
+          <t>$226228    0.0
+INSTALATII SANITARE OB.2 e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
         </is>
       </c>
       <c r="D262" s="9" t="inlineStr">
@@ -5960,8 +5960,8 @@
       </c>
       <c r="C263" s="8" t="inlineStr">
         <is>
-          <t>$3210241  buc  4.0
-Teu egal PPR 32</t>
+          <t>$05024  buc  3.0
+MONTAT DUS GRUP SANITAR material: manopera: utilaj: transport:</t>
         </is>
       </c>
       <c r="D263" s="9" t="inlineStr">
@@ -5981,8 +5981,8 @@
       </c>
       <c r="C264" s="8" t="inlineStr">
         <is>
-          <t>$226428    0.0
-INSTALATII SANITARE OB 4 e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
+          <t>$22222242  buc  9.0
+Oglinda cu rama aluminiu</t>
         </is>
       </c>
       <c r="D264" s="9" t="inlineStr">
@@ -6023,8 +6023,8 @@
       </c>
       <c r="C266" s="8" t="inlineStr">
         <is>
-          <t>$32719861  buc  3.0
-ROBINET SFERA APA 1"GIACOMINI DN 25 R</t>
+          <t>$3210241  buc  4.0
+Teu egal PPR 32</t>
         </is>
       </c>
       <c r="D266" s="9" t="inlineStr">
@@ -6044,8 +6044,8 @@
       </c>
       <c r="C267" s="8" t="inlineStr">
         <is>
-          <t>$3211097  buc  4.0
-REDUCTIE PPR 40-32</t>
+          <t>$32719871  buc  3.0
+ROBINET SFERA APA 1"1/4 GIACOMINI DN 32 R 250</t>
         </is>
       </c>
       <c r="D267" s="9" t="inlineStr">
@@ -6086,8 +6086,8 @@
       </c>
       <c r="C269" s="8" t="inlineStr">
         <is>
-          <t>$05022  buc  7.0
-MONTAT WC GRUP SANITAR material: manopera: utilaj: transport:</t>
+          <t>$2222219  buc  3.0
+CADITE DUS</t>
         </is>
       </c>
       <c r="D269" s="9" t="inlineStr">
@@ -6107,8 +6107,8 @@
       </c>
       <c r="C270" s="8" t="inlineStr">
         <is>
-          <t>$327101  m  35.7
-TEAVA PN20 PPR VERDE DN32</t>
+          <t>$3211097  buc  4.0
+REDUCTIE PPR 40-32</t>
         </is>
       </c>
       <c r="D270" s="9" t="inlineStr">
@@ -6128,8 +6128,8 @@
       </c>
       <c r="C271" s="8" t="inlineStr">
         <is>
-          <t>$226528    0.0
-INSTALATII SANITARE OB 5 e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
+          <t>$05022  buc  7.0
+MONTAT WC GRUP SANITAR material: manopera: utilaj: transport:</t>
         </is>
       </c>
       <c r="D271" s="9" t="inlineStr">
@@ -6149,8 +6149,8 @@
       </c>
       <c r="C272" s="8" t="inlineStr">
         <is>
-          <t>$05024  buc  3.0
-MONTAT DUS GRUP SANITAR material: manopera: utilaj: transport:</t>
+          <t>$226528    0.0
+INSTALATII SANITARE OB 5 e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
         </is>
       </c>
       <c r="D272" s="9" t="inlineStr">
@@ -6170,8 +6170,8 @@
       </c>
       <c r="C273" s="8" t="inlineStr">
         <is>
-          <t>$22222242  buc  9.0
-Oglinda cu rama aluminiu</t>
+          <t>$327101  m  35.7
+TEAVA PN20 PPR VERDE DN32</t>
         </is>
       </c>
       <c r="D273" s="9" t="inlineStr">
@@ -6556,8 +6556,8 @@
       </c>
       <c r="C292" s="8" t="inlineStr">
         <is>
-          <t>$6311528  kg  15.3
-Scoaba otel pentru constructii din lemn, latime= 65-90MM, L.200-300 MM Greutate Materiale (tone) Ore Manopera Material Manopera Utilaj Transport TOTAL Deviz "226508" - Formular F3 Formular generat cu programul @Devize (www.eDevize.ro) Pagina 5 din 6</t>
+          <t>$226508    0.0
+STRUCTURA DE REZISTENTA(GRUPURI SANITARE PUBLICE) e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
         </is>
       </c>
       <c r="D292" s="9" t="inlineStr">
@@ -6577,8 +6577,8 @@
       </c>
       <c r="C293" s="8" t="inlineStr">
         <is>
-          <t>$226508    0.0
-STRUCTURA DE REZISTENTA(GRUPURI SANITARE PUBLICE) e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
+          <t>$32745863  kg  1344.88
+OTEL BETON BST500 10-16</t>
         </is>
       </c>
       <c r="D293" s="9" t="inlineStr">
@@ -6598,8 +6598,8 @@
       </c>
       <c r="C294" s="8" t="inlineStr">
         <is>
-          <t>$32745863  kg  1344.88
-OTEL BETON BST500 10-16</t>
+          <t>$32745843  kg  319.73
+OTEL BETON BST500 6-8</t>
         </is>
       </c>
       <c r="D294" s="9" t="inlineStr">
@@ -6619,8 +6619,8 @@
       </c>
       <c r="C295" s="8" t="inlineStr">
         <is>
-          <t>$32745843  kg  319.73
-OTEL BETON BST500 6-8</t>
+          <t>$6311528  kg  15.3
+Scoaba otel pentru constructii din lemn, latime= 65-90MM, L.200-300 MM Greutate Materiale (tone) Ore Manopera Material Manopera Utilaj Transport TOTAL Deviz "226508" - Formular F3 Formular generat cu programul @Devize (www.eDevize.ro) Pagina 5 din 6</t>
         </is>
       </c>
       <c r="D295" s="9" t="inlineStr">
@@ -6934,8 +6934,8 @@
       </c>
       <c r="C310" s="8" t="inlineStr">
         <is>
-          <t>$71100111  m  6.0
-@BURLAN DIN TABLA VOPSITA ELECTROSTATIC DE DN=15 CM</t>
+          <t>$226518    0.0
+ARHITECTURA GRUPURI SANITARE PUBLICE e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
         </is>
       </c>
       <c r="D310" s="9" t="inlineStr">
@@ -6955,8 +6955,8 @@
       </c>
       <c r="C311" s="8" t="inlineStr">
         <is>
-          <t>$71100101  m  7.0
-@JGHEAB TABLA VOPSITA ELECTROSTATIC DE 15 CM</t>
+          <t>$4741  kg  384.0
+71</t>
         </is>
       </c>
       <c r="D311" s="9" t="inlineStr">
@@ -6976,8 +6976,8 @@
       </c>
       <c r="C312" s="8" t="inlineStr">
         <is>
-          <t>$32742701  kg  11.5
-Adeziv granit</t>
+          <t>$16509  mp  120.0
+VOPSITORIE DECORATIVA material: manopera: utilaj: transport: Deviz "226518" - Formular F3 Formular generat cu programul @Devize (www.eDevize.ro) Pagina 2 din 7</t>
         </is>
       </c>
       <c r="D312" s="9" t="inlineStr">
@@ -6997,8 +6997,8 @@
       </c>
       <c r="C313" s="8" t="inlineStr">
         <is>
-          <t>PF04A1ASIM  mp  24.0
-STRAT AMORSAJ APLICAT CU PERIA DIN BITUM TAIAT CU WHITE SPIRIT RAFINAT</t>
+          <t>$7800774  mp  61.71
+Folie anticondens</t>
         </is>
       </c>
       <c r="D313" s="9" t="inlineStr">
@@ -7018,8 +7018,8 @@
       </c>
       <c r="C314" s="8" t="inlineStr">
         <is>
-          <t>$6306493  mp  15.0
-USA PVC</t>
+          <t>$71100111  m  6.0
+@BURLAN DIN TABLA VOPSITA ELECTROSTATIC DE DN=15 CM</t>
         </is>
       </c>
       <c r="D314" s="9" t="inlineStr">
@@ -7039,8 +7039,8 @@
       </c>
       <c r="C315" s="8" t="inlineStr">
         <is>
-          <t>$32750461  mp  48.0
-VATA MINERALA 10 cm</t>
+          <t>$22041951  m  9.0
+GLAF EXT TABLA VOPSITA 25 CM, CU PICURATOR SI ACCESORII PE MONTAJ</t>
         </is>
       </c>
       <c r="D315" s="9" t="inlineStr">
@@ -7060,8 +7060,8 @@
       </c>
       <c r="C316" s="8" t="inlineStr">
         <is>
-          <t>$7800859  kg  12.0
-Vopsea lavabila acrilica</t>
+          <t>$6306493  mp  15.0
+USA PVC</t>
         </is>
       </c>
       <c r="D316" s="9" t="inlineStr">
@@ -7081,8 +7081,8 @@
       </c>
       <c r="C317" s="8" t="inlineStr">
         <is>
-          <t>$226518    0.0
-ARHITECTURA GRUPURI SANITARE PUBLICE e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
+          <t>PF04A1ASIM  mp  24.0
+STRAT AMORSAJ APLICAT CU PERIA DIN BITUM TAIAT CU WHITE SPIRIT RAFINAT</t>
         </is>
       </c>
       <c r="D317" s="9" t="inlineStr">
@@ -7102,7 +7102,8 @@
       </c>
       <c r="C318" s="8" t="inlineStr">
         <is>
-          <t>S7064  kg  22.5</t>
+          <t>$32742701  kg  11.5
+Adeziv granit</t>
         </is>
       </c>
       <c r="D318" s="9" t="inlineStr">
@@ -7122,8 +7123,8 @@
       </c>
       <c r="C319" s="8" t="inlineStr">
         <is>
-          <t>$22041951  m  9.0
-GLAF EXT TABLA VOPSITA 25 CM, CU PICURATOR SI ACCESORII PE MONTAJ</t>
+          <t>$16508  mp  120.0
+SISTEM TERMOIZ. CU VATA MINERALA B material: manopera: utilaj: transport:</t>
         </is>
       </c>
       <c r="D319" s="9" t="inlineStr">
@@ -7143,8 +7144,8 @@
       </c>
       <c r="C320" s="8" t="inlineStr">
         <is>
-          <t>$16509  mp  120.0
-VOPSITORIE DECORATIVA material: manopera: utilaj: transport: Deviz "226518" - Formular F3 Formular generat cu programul @Devize (www.eDevize.ro) Pagina 2 din 7</t>
+          <t>$7800859  kg  12.0
+Vopsea lavabila acrilica</t>
         </is>
       </c>
       <c r="D320" s="9" t="inlineStr">
@@ -7164,8 +7165,7 @@
       </c>
       <c r="C321" s="8" t="inlineStr">
         <is>
-          <t>$7800774  mp  61.71
-Folie anticondens</t>
+          <t>S7064  kg  22.5</t>
         </is>
       </c>
       <c r="D321" s="9" t="inlineStr">
@@ -7185,8 +7185,8 @@
       </c>
       <c r="C322" s="8" t="inlineStr">
         <is>
-          <t>$4741  kg  384.0
-71</t>
+          <t>$32750461  mp  48.0
+VATA MINERALA 10 cm</t>
         </is>
       </c>
       <c r="D322" s="9" t="inlineStr">
@@ -7206,8 +7206,8 @@
       </c>
       <c r="C323" s="8" t="inlineStr">
         <is>
-          <t>$16508  mp  120.0
-SISTEM TERMOIZ. CU VATA MINERALA B material: manopera: utilaj: transport:</t>
+          <t>$71100101  m  7.0
+@JGHEAB TABLA VOPSITA ELECTROSTATIC DE 15 CM</t>
         </is>
       </c>
       <c r="D323" s="9" t="inlineStr">
@@ -7699,8 +7699,8 @@
       </c>
       <c r="C346" s="8" t="inlineStr">
         <is>
-          <t>$32723641  buc  4.0
-VAS WC</t>
+          <t>$05022  buc  4.0
+MONTAT WC GRUP SANITAR material: manopera: utilaj: transport: Deviz "226528" - Formular F3 Formular generat cu programul @Devize (www.eDevize.ro) Pagina 9 din 12</t>
         </is>
       </c>
       <c r="D346" s="9" t="inlineStr">
@@ -7720,8 +7720,8 @@
       </c>
       <c r="C347" s="8" t="inlineStr">
         <is>
-          <t>SD13A1  buc  4.0
-Robinet trec. cu ventil si mufe, pentru tevi otel cu D= 1/2 sau D= 3/8 toli material: manopera: utilaj: transport:</t>
+          <t>$32723641  buc  4.0
+VAS WC</t>
         </is>
       </c>
       <c r="D347" s="9" t="inlineStr">
@@ -7741,8 +7741,8 @@
       </c>
       <c r="C348" s="8" t="inlineStr">
         <is>
-          <t>$22222131  buc  1.0
-PERIE WC</t>
+          <t>$327101  m  5.0
+TEAVA PN20 PPR VERDE DN32</t>
         </is>
       </c>
       <c r="D348" s="9" t="inlineStr">
@@ -7762,8 +7762,8 @@
       </c>
       <c r="C349" s="8" t="inlineStr">
         <is>
-          <t>$05021  buc  4.0
-MONTAT LAVOAR GRUP SANITAR material: manopera: utilaj: transport:</t>
+          <t>$3211097  buc  1.0
+REDUCTIE PPR 40-32</t>
         </is>
       </c>
       <c r="D349" s="9" t="inlineStr">
@@ -7783,7 +7783,8 @@
       </c>
       <c r="C350" s="8" t="inlineStr">
         <is>
-          <t>S9610  buc  1.0</t>
+          <t>$22222121  buc  1.0
+SUPORT HARTIE IGIENICA</t>
         </is>
       </c>
       <c r="D350" s="9" t="inlineStr">
@@ -7824,8 +7825,8 @@
       </c>
       <c r="C352" s="8" t="inlineStr">
         <is>
-          <t>$22222121  buc  1.0
-SUPORT HARTIE IGIENICA</t>
+          <t>$05027  buc  1.0
+MONTAT WC PERSOANE CU DIZABILITATI material: manopera: utilaj: transport:</t>
         </is>
       </c>
       <c r="D352" s="9" t="inlineStr">
@@ -7845,8 +7846,7 @@
       </c>
       <c r="C353" s="8" t="inlineStr">
         <is>
-          <t>$3271744  buc  4.0
-COT PP D 110X45</t>
+          <t>S9610  buc  1.0</t>
         </is>
       </c>
       <c r="D353" s="9" t="inlineStr">
@@ -7866,8 +7866,8 @@
       </c>
       <c r="C354" s="8" t="inlineStr">
         <is>
-          <t>$3210241  buc  1.0
-Teu egal PPR 32</t>
+          <t>$32719861  buc  1.0
+ROBINET SFERA APA 1"GIACOMINI DN 25 R</t>
         </is>
       </c>
       <c r="D354" s="9" t="inlineStr">
@@ -7887,8 +7887,8 @@
       </c>
       <c r="C355" s="8" t="inlineStr">
         <is>
-          <t>$22222241  buc  1.0
-Oglinda</t>
+          <t>$05021  buc  4.0
+MONTAT LAVOAR GRUP SANITAR material: manopera: utilaj: transport:</t>
         </is>
       </c>
       <c r="D355" s="9" t="inlineStr">
@@ -7908,8 +7908,8 @@
       </c>
       <c r="C356" s="8" t="inlineStr">
         <is>
-          <t>$05027  buc  1.0
-MONTAT WC PERSOANE CU DIZABILITATI material: manopera: utilaj: transport:</t>
+          <t>$3210241  buc  1.0
+Teu egal PPR 32</t>
         </is>
       </c>
       <c r="D356" s="9" t="inlineStr">
@@ -7929,8 +7929,8 @@
       </c>
       <c r="C357" s="8" t="inlineStr">
         <is>
-          <t>$05028  buc  1.0
-MONTAT LAVOAR PERSOANE CU DIZABILITATI material: manopera: utilaj: transport:</t>
+          <t>$3271744  buc  4.0
+COT PP D 110X45</t>
         </is>
       </c>
       <c r="D357" s="9" t="inlineStr">
@@ -7950,8 +7950,8 @@
       </c>
       <c r="C358" s="8" t="inlineStr">
         <is>
-          <t>$05022  buc  4.0
-MONTAT WC GRUP SANITAR material: manopera: utilaj: transport: Deviz "226528" - Formular F3 Formular generat cu programul @Devize (www.eDevize.ro) Pagina 9 din 12</t>
+          <t>$22222131  buc  1.0
+PERIE WC</t>
         </is>
       </c>
       <c r="D358" s="9" t="inlineStr">
@@ -7971,8 +7971,8 @@
       </c>
       <c r="C359" s="8" t="inlineStr">
         <is>
-          <t>$32719861  buc  1.0
-ROBINET SFERA APA 1"GIACOMINI DN 25 R</t>
+          <t>$22222242  buc  4.0
+Oglinda cu rama aluminiu</t>
         </is>
       </c>
       <c r="D359" s="9" t="inlineStr">
@@ -7992,8 +7992,8 @@
       </c>
       <c r="C360" s="8" t="inlineStr">
         <is>
-          <t>$327101  m  5.0
-TEAVA PN20 PPR VERDE DN32</t>
+          <t>SD13A1  buc  4.0
+Robinet trec. cu ventil si mufe, pentru tevi otel cu D= 1/2 sau D= 3/8 toli material: manopera: utilaj: transport:</t>
         </is>
       </c>
       <c r="D360" s="9" t="inlineStr">
@@ -8013,8 +8013,8 @@
       </c>
       <c r="C361" s="8" t="inlineStr">
         <is>
-          <t>$3211097  buc  1.0
-REDUCTIE PPR 40-32</t>
+          <t>$22222241  buc  1.0
+Oglinda</t>
         </is>
       </c>
       <c r="D361" s="9" t="inlineStr">
@@ -8034,8 +8034,8 @@
       </c>
       <c r="C362" s="8" t="inlineStr">
         <is>
-          <t>$22222242  buc  4.0
-Oglinda cu rama aluminiu</t>
+          <t>$05028  buc  1.0
+MONTAT LAVOAR PERSOANE CU DIZABILITATI material: manopera: utilaj: transport:</t>
         </is>
       </c>
       <c r="D362" s="9" t="inlineStr">
@@ -8188,8 +8188,8 @@
       </c>
       <c r="C370" s="8" t="inlineStr">
         <is>
-          <t>$226478    0.0
-INSTALATII ELECTRICE CURENTI TARI OB 4 e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
+          <t>W1MM05A  buc  1.0
+Masurarea rezistentei prizei de legare la pamant .</t>
         </is>
       </c>
       <c r="D370" s="9" t="inlineStr">
@@ -8209,8 +8209,8 @@
       </c>
       <c r="C371" s="8" t="inlineStr">
         <is>
-          <t>W1MM05A  buc  1.0
-Masurarea rezistentei prizei de legare la pamant .</t>
+          <t>$226558    0.0
+INSTALATII ELECTRICE CURENTI TARI OB 5 e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
         </is>
       </c>
       <c r="D371" s="9" t="inlineStr">
@@ -8230,8 +8230,8 @@
       </c>
       <c r="C372" s="8" t="inlineStr">
         <is>
-          <t>W1MM05A  buc  1.0
-Masurarea rezistentei prizei de legare la pamant .</t>
+          <t>$226478    0.0
+INSTALATII ELECTRICE CURENTI TARI OB 4 e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
         </is>
       </c>
       <c r="D372" s="9" t="inlineStr">
@@ -8251,8 +8251,8 @@
       </c>
       <c r="C373" s="8" t="inlineStr">
         <is>
-          <t>$226558    0.0
-INSTALATII ELECTRICE CURENTI TARI OB 5 e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
+          <t>W1MM05A  buc  1.0
+Masurarea rezistentei prizei de legare la pamant .</t>
         </is>
       </c>
       <c r="D373" s="9" t="inlineStr">
@@ -8913,8 +8913,8 @@
       </c>
       <c r="C407" s="8" t="inlineStr">
         <is>
-          <t>IZD04D1  tona  8.0
-Vopsire cu aparat aer compr vopsea ulei pe conf siconstr met profile 8-12MM 2straturi material: manopera: utilaj: transport: Deviz "226328" - Formular F3 Formular generat cu programul @Devize (www.eDevize.ro) Pagina 1 din 2</t>
+          <t>$36448571  mp  590.515
+Panou cutat zincat</t>
         </is>
       </c>
       <c r="D407" s="9" t="inlineStr">
@@ -8934,8 +8934,8 @@
       </c>
       <c r="C408" s="8" t="inlineStr">
         <is>
-          <t>$36448571  mp  590.515
-Panou cutat zincat</t>
+          <t>IZD03D1  tona  8.0
+Vopsire cu vops miniu cu aparat aer compr 1 str peconf si ctii metal exec din prof gros 8-12 MM material: manopera: utilaj: transport:</t>
         </is>
       </c>
       <c r="D408" s="9" t="inlineStr">
@@ -8955,8 +8955,8 @@
       </c>
       <c r="C409" s="8" t="inlineStr">
         <is>
-          <t>$226328    0.0
-ARHITECTURA GRADENE e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
+          <t>IZD04D1  tona  8.0
+Vopsire cu aparat aer compr vopsea ulei pe conf siconstr met profile 8-12MM 2straturi material: manopera: utilaj: transport: Deviz "226328" - Formular F3 Formular generat cu programul @Devize (www.eDevize.ro) Pagina 1 din 2</t>
         </is>
       </c>
       <c r="D409" s="9" t="inlineStr">
@@ -8976,8 +8976,8 @@
       </c>
       <c r="C410" s="8" t="inlineStr">
         <is>
-          <t>IZD03D1  tona  8.0
-Vopsire cu vops miniu cu aparat aer compr 1 str peconf si ctii metal exec din prof gros 8-12 MM material: manopera: utilaj: transport:</t>
+          <t>$226328    0.0
+ARHITECTURA GRADENE e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
         </is>
       </c>
       <c r="D410" s="9" t="inlineStr">
@@ -9095,8 +9095,8 @@
       </c>
       <c r="C417" s="8" t="inlineStr">
         <is>
-          <t>$226038    0.0
-TELECOMUNICATII e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
+          <t>$226488    0.0
+INSTALATIE VOCE DATE OB 4 e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
         </is>
       </c>
       <c r="D417" s="9" t="inlineStr">
@@ -9116,8 +9116,8 @@
       </c>
       <c r="C418" s="8" t="inlineStr">
         <is>
-          <t>$226488    0.0
-INSTALATIE VOCE DATE OB 4 e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
+          <t>$226568    0.0
+INSTALATIE VOCE DATE OB 5 e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
         </is>
       </c>
       <c r="D418" s="9" t="inlineStr">
@@ -9137,8 +9137,8 @@
       </c>
       <c r="C419" s="8" t="inlineStr">
         <is>
-          <t>$226578    0.0
-SISTEM SUPRAVEGHERE VIDEO OB 5 e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
+          <t>$226038    0.0
+TELECOMUNICATII e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
         </is>
       </c>
       <c r="D419" s="9" t="inlineStr">
@@ -9179,8 +9179,8 @@
       </c>
       <c r="C421" s="8" t="inlineStr">
         <is>
-          <t>$226568    0.0
-INSTALATIE VOCE DATE OB 5 e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
+          <t>$226498    0.0
+SISTEM SUPRAVEGHERE VIDEO e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
         </is>
       </c>
       <c r="D421" s="9" t="inlineStr">
@@ -9200,8 +9200,8 @@
       </c>
       <c r="C422" s="8" t="inlineStr">
         <is>
-          <t>$226498    0.0
-SISTEM SUPRAVEGHERE VIDEO e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
+          <t>EA02A2  m  100.0
+Tub izolant, de protectie, etans, ipe, din policlorura de vinil neplastifiata, ipey, montat ingropat sau aparent, avand diametrul exterior de 20 MM, montat ingropat</t>
         </is>
       </c>
       <c r="D422" s="9" t="inlineStr">
@@ -9221,8 +9221,8 @@
       </c>
       <c r="C423" s="8" t="inlineStr">
         <is>
-          <t>EA02A2  m  100.0
-Tub izolant, de protectie, etans, ipe, din policlorura de vinil neplastifiata, ipey, montat ingropat sau aparent, avand diametrul exterior de 20 MM, montat ingropat</t>
+          <t>$226578    0.0
+SISTEM SUPRAVEGHERE VIDEO OB 5 e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
         </is>
       </c>
       <c r="D423" s="9" t="inlineStr">
@@ -9479,7 +9479,7 @@
     <row r="439" ht="20" customHeight="1">
       <c r="A439" s="6" t="inlineStr">
         <is>
-          <t>Categoria de lucrari: ALIMENTARE CU APA</t>
+          <t>Categoria de lucrari: INSTALATIE VENTILATIE OB 4 e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar (fara TVA) - Lei - TOTALUL (fara TVA) - Lei - 0 1 2 3 4 5 = 3 x 4 1 VC01C1 - Montarea ventilatorului axial GR. totala 50- 200Kg buc 4.000 325.09 1,300.38 material: 102.34 409.38 manopera: 222.75 891.00 utilaj: 0.00 0.00 transport: 0.00 0.00 1 3270546 - VENTILATOR BAIE D=100MM, MODEL "EOL 100T" TIMER buc 3.000 178.00 534.00 1 3272502 - VENTILATOR BAIE SILENT-100CZ-D=100-230V- 95MC/H-SOLER PALAU buc 1.000 225.00 225.00 2 VB14D1 - Priza de aer det tip 61/105 avind perimetrul 1401-2500 MM montata pe canal buc 1.000 71.47 71.47 material: 32.78 32.78 manopera: 38.70 38.70 utilaj: 0.00 0.00 transport: 0.00 0.00 2 7002221 - GRILA VENTILATIE DN110 MM BUC 1.000 135.00 135.00 3 VB14D1 - Priza de aer det tip 61/105 avind perimetrul 1401-2500 MM montata pe canal buc 2.000 71.47 142.95 material: 32.78 65.55 manopera: 38.70 77.40 utilaj: 0.00 0.00 transport: 0.00 0.00 3 2997228 - GRILA EXTERIOARA CU JALUZELE FIXE Dn125 cu jaluzele anti ploaie si plasa antiinsecte buc 2.000 35.00 70.00 4 VB30A1 - Anemostat plan patrat det tip 61/272 buc 4.000 69.78 279.14 material: 6.78 27.14 manopera: 63.00 252.00 utilaj: 0.00 0.00 transport: 0.00 0.00 4 2997173 - GRILA TRANSFER CU IZOLARE FONICA, ALUMINIU MONTAT IN USA 300X200 INCLUSIV CONTRARAMA buc 4.000 185.00 740.00 5 VA02B08 - Canale drepte confectionata pe sant cu perim sect de 400- 700 mm cu sect circ din tabla zinc de 0. 5 mm mp 4.500 165.79 746.07 material: 97.99 440.97 manopera: 67.80 305.10 utilaj: 0.00 0.00 transport: 0.00 0.00 Deviz "226448" - Formular F3 Formular generat cu programul @Devize (www.eDevize.ro) Pagina 1 din 2</t>
         </is>
       </c>
     </row>
@@ -9494,8 +9494,8 @@
       </c>
       <c r="C440" s="8" t="inlineStr">
         <is>
-          <t>$6716997  m  345.0
-BANDA PVC CU INSERTIE DE METAL DETECTABIL</t>
+          <t>$1401  buc  2.0
+2500 MM montata pe canal material: manopera: utilaj: transport:</t>
         </is>
       </c>
       <c r="D440" s="9" t="inlineStr">
@@ -9515,8 +9515,8 @@
       </c>
       <c r="C441" s="8" t="inlineStr">
         <is>
-          <t>TRI1AA01C2  tona  117.8
-Incarcarea materialelor, grupa a-grele si marunte,prin aruncare rampa sau teren-auto categ.2</t>
+          <t>$226448    0.0
+INSTALATIE VENTILATIE OB 4 e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
         </is>
       </c>
       <c r="D441" s="9" t="inlineStr">
@@ -9528,7 +9528,7 @@
     <row r="442" ht="20" customHeight="1">
       <c r="A442" s="6" t="inlineStr">
         <is>
-          <t>Categoria de lucrari: INSTAI.ATII VENTILATIE OB.2 eDevize e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar (fara TVA) - Lei - TOTALUL (fara TVA) - Lei - 0 1 2 3 4 5 = 3 x 4 1 VC01C1 - Montarea ventilatorului axial GR. totala 50- 200Kg buc 4.000 325.09 1,300.38 material: 102.34 409.38 manopera: 222.75 891.00 utilaj: 0.00 0.00 transport: 0.00 0.00 1 3270546 - VENTILATOR BAIE D=100MM, MODEL "EOL 100T" TIMER buc 4.000 178.00 712.00 2 VB14D1 - Priza de aer det tip 61/105 avind perimetrul 1401-2500 MM montata pe canal buc 4.000 71.47 285.90 material: 32.78 131.10 manopera: 38.70 154.80 utilaj: 0.00 0.00 transport: 0.00 0.00 2 7002221 - GRILA VENTILATIE DN110 MM BUC 4.000 135.00 540.00 3 VB30A1 - Anemostat plan patrat det tip 61/272 buc 4.000 69.78 279.14 material: 6.78 27.14 manopera: 63.00 252.00 utilaj: 0.00 0.00 transport: 0.00 0.00 3 2997173 - GRILA TRANSFER CU IZOLARE FONICA, ALUMINIU MONTAT IN USA 300X200 INCLUSIV CONTRARAMA buc 4.000 185.00 740.00 4 VA02B08 - Canale drepte confectionata pe sant cu perim sect de 400- 700 mm cu sect circ din tabla zinc de 0. 5 mm mp 5.000 165.79 828.96 material: 97.99 489.96 manopera: 67.80 339.00 utilaj: 0.00 0.00 transport: 0.00 0.00 4 7000777 - TUBUILATURA CIRCULARA RIGIDA D=100 NEIZOLATA, INCLUSIV PIESE SPECIALA SI SUPORTI SUPORT X m 15.000 35.00 525.00 5 VC23A1 - Confectionare dispoz. sust-ancor. pentru aparate canale piese spec. din otel prof. greut/buc sub 5 Kg. kg 10.000 26.70 266.99 material: 10.53 105.29 manopera: 16.17 161.69 utilaj: 0.00 0.00 transport: 0.00 0.00 Deviz "226248" - Formular F3 Formular generat cu programul @Devize (www.eDevize.ro) Pagina 1 din 2</t>
+          <t>Categoria de lucrari: INSTALATII VENTILATIE OB. 4</t>
         </is>
       </c>
     </row>
@@ -9543,8 +9543,8 @@
       </c>
       <c r="C443" s="8" t="inlineStr">
         <is>
-          <t>$226248    0.0
-INSTAI.ATII VENTILATIE OB.2 eDevize e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
+          <t>$1401  buc  2.0
+2500 MM montata pe canal material: manopera: utilaj: transport:</t>
         </is>
       </c>
       <c r="D443" s="9" t="inlineStr">
@@ -9564,8 +9564,8 @@
       </c>
       <c r="C444" s="8" t="inlineStr">
         <is>
-          <t>$1401  buc  4.0
-2500 MM montata pe canal material: manopera: utilaj: transport:</t>
+          <t>$226538    0.0
+INSTALATII VENTILATIE OB 5 e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
         </is>
       </c>
       <c r="D444" s="9" t="inlineStr">
@@ -9577,7 +9577,7 @@
     <row r="445" ht="20" customHeight="1">
       <c r="A445" s="6" t="inlineStr">
         <is>
-          <t>Categoria de lucrari: MONTAJ SISTEM PANOU FOTOVOLTAICE</t>
+          <t>Categoria de lucrari: TELECOMUNICATII</t>
         </is>
       </c>
     </row>
@@ -9592,8 +9592,8 @@
       </c>
       <c r="C446" s="8" t="inlineStr">
         <is>
-          <t>$32745841  kg  1979.25
-OTEL BETON BST500 6-8 mm (BARA) 12 M</t>
+          <t>TRI1AA01C2  tona  8.42
+Incarcarea materialelor, grupa a-grele si marunte, prin aruncare rampa sau teren-auto categ.2</t>
         </is>
       </c>
       <c r="D446" s="9" t="inlineStr">
@@ -9613,7 +9613,8 @@
       </c>
       <c r="C447" s="8" t="inlineStr">
         <is>
-          <t>S7064  kg  45.0</t>
+          <t>W2H04A1  mc  16.0
+Strat nisip asezat in sant pentru protejarea cablurilor la lucr in prof netipizat material: manopera: utilaj: transport:</t>
         </is>
       </c>
       <c r="D447" s="9" t="inlineStr">
@@ -9633,8 +9634,8 @@
       </c>
       <c r="C448" s="8" t="inlineStr">
         <is>
-          <t>$32745861  kg  2324.35
-OTEL BETON BST500 10-12 mm (BARA) 12 M</t>
+          <t>$67185061  m  200.0
+BANDA AVERTIZOARE PVC INSCRIPTIONATA PENTRU CABLU TELECOMUNICATII ÎN SAPATURA 1 MM GROSIME</t>
         </is>
       </c>
       <c r="D448" s="9" t="inlineStr">
@@ -9643,31 +9644,31 @@
         </is>
       </c>
     </row>
-    <row r="449" ht="40" customHeight="1">
-      <c r="A449" s="7" t="n">
+    <row r="449" ht="20" customHeight="1">
+      <c r="A449" s="6" t="inlineStr">
+        <is>
+          <t>Categoria de lucrari: ALIMENTARE CU E.E, SI ILUMINAT EXTERIOR</t>
+        </is>
+      </c>
+    </row>
+    <row r="450" ht="40" customHeight="1">
+      <c r="A450" s="7" t="n">
         <v>410</v>
       </c>
-      <c r="B449" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C449" s="8" t="inlineStr">
-        <is>
-          <t>W1C01A1  buc  1.0
-ASIMILAT - MONTARE PANOURI FOTOVOLTAICE</t>
-        </is>
-      </c>
-      <c r="D449" s="9" t="inlineStr">
-        <is>
-          <t>ARTICOL SUPLIMENTAR ÎN OFERTĂ</t>
-        </is>
-      </c>
-    </row>
-    <row r="450" ht="20" customHeight="1">
-      <c r="A450" s="6" t="inlineStr">
-        <is>
-          <t>Categoria de lucrari: ALIMENTARE CU E.E, SI ILUMINAT EXTERIOR</t>
+      <c r="B450" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C450" s="8" t="inlineStr">
+        <is>
+          <t>W2F05C01  buc  4.0
+Corp de ilum. publ. tip lampadar pentru lampa cu vap. me rcur inal. pres. cu scara manuale pe st. metal montat</t>
+        </is>
+      </c>
+      <c r="D450" s="9" t="inlineStr">
+        <is>
+          <t>ARTICOL SUPLIMENTAR ÎN OFERTĂ</t>
         </is>
       </c>
     </row>
@@ -9682,8 +9683,8 @@
       </c>
       <c r="C451" s="8" t="inlineStr">
         <is>
-          <t>$7319524  m  128.52
-Electrod teava zincata 76,1X4,5</t>
+          <t>W1MN14C  m  126.0
+Electrod din teava de otel zincata pentru priza de legare la pamant teren foarte tare</t>
         </is>
       </c>
       <c r="D451" s="9" t="inlineStr">
@@ -9703,8 +9704,8 @@
       </c>
       <c r="C452" s="8" t="inlineStr">
         <is>
-          <t>W2E12J01  buc  1.0
-Tablou distrib mod ideb Montare firida sig mpr 315-630 a tip 4e-5b cu5 set mpr 6 sig lfd-iii</t>
+          <t>W2A16A1  buc  38.0
+Stalp simplu teava otel in fundatie turnata teren N0rmal</t>
         </is>
       </c>
       <c r="D452" s="9" t="inlineStr">
@@ -9724,8 +9725,8 @@
       </c>
       <c r="C453" s="8" t="inlineStr">
         <is>
-          <t>W1MN06A  buc  38.0
-Piesa de separatie pentru priza de pamant - montare -</t>
+          <t>W2G02B31  m  100.0
+Montare cablu subt. 1 kv gr 2,901-3,200 kg/m cu-al in tub pe traseu cu obst. tr. manuala montat</t>
         </is>
       </c>
       <c r="D453" s="9" t="inlineStr">
@@ -9745,8 +9746,8 @@
       </c>
       <c r="C454" s="8" t="inlineStr">
         <is>
-          <t>W1F12D  buc  1.0
-Incercari pentru masurarea tensiunii de atingere si de pas.</t>
+          <t>W2H04A1  mc  68.0
+Strat nisip asezat in sant pentru protejarea cablurilor la lucr in prof netipizat</t>
         </is>
       </c>
       <c r="D454" s="9" t="inlineStr">
@@ -9766,8 +9767,8 @@
       </c>
       <c r="C455" s="8" t="inlineStr">
         <is>
-          <t>W2H04A1  mc  68.0
-Strat nisip asezat in sant pentru protejarea cablurilor la lucr in prof netipizat</t>
+          <t>W3E06A1  buc  10.0
+Masurarea tensiunilor de atingere si pas la l. c.</t>
         </is>
       </c>
       <c r="D455" s="9" t="inlineStr">
@@ -9787,8 +9788,8 @@
       </c>
       <c r="C456" s="8" t="inlineStr">
         <is>
-          <t>$3275630  m  100.0
-CABLURI ELECTRICE CYABY-F 3X95+50 , 71760471360100 ICME ECAB</t>
+          <t>$7319524  m  128.52
+Electrod teava zincata 76,1X4,5</t>
         </is>
       </c>
       <c r="D456" s="9" t="inlineStr">
@@ -9808,8 +9809,8 @@
       </c>
       <c r="C457" s="8" t="inlineStr">
         <is>
-          <t>W2F05C01  buc  4.0
-Corp de ilum. publ. tip lampadar pentru lampa cu vap. me rcur inal. pres. cu scara manuale pe st. metal montat</t>
+          <t>W1MN06A  buc  38.0
+Piesa de separatie pentru priza de pamant - montare -</t>
         </is>
       </c>
       <c r="D457" s="9" t="inlineStr">
@@ -9829,8 +9830,8 @@
       </c>
       <c r="C458" s="8" t="inlineStr">
         <is>
-          <t>W2G02B31  m  100.0
-Montare cablu subt. 1 kv gr 2,901-3,200 kg/m cu-al in tub pe traseu cu obst. tr. manuala montat</t>
+          <t>W1F12D  buc  1.0
+Incercari pentru masurarea tensiunii de atingere si de pas.</t>
         </is>
       </c>
       <c r="D458" s="9" t="inlineStr">
@@ -9850,8 +9851,8 @@
       </c>
       <c r="C459" s="8" t="inlineStr">
         <is>
-          <t>W1MN14C  m  126.0
-Electrod din teava de otel zincata pentru priza de legare la pamant teren foarte tare</t>
+          <t>W2G01B19  m  800.0
+Montare cablu U1KV gr 1,301-1,500 Kg/M cu sau al sant pat nisip cu obstac cu tract manuala</t>
         </is>
       </c>
       <c r="D459" s="9" t="inlineStr">
@@ -9871,8 +9872,8 @@
       </c>
       <c r="C460" s="8" t="inlineStr">
         <is>
-          <t>W3E06A1  buc  10.0
-Masurarea tensiunilor de atingere si pas la l. c.</t>
+          <t>W2E12J01  buc  1.0
+Tablou distrib mod ideb Montare firida sig mpr 315-630 a tip 4e-5b cu5 set mpr 6 sig lfd-iii</t>
         </is>
       </c>
       <c r="D460" s="9" t="inlineStr">
@@ -9892,8 +9893,8 @@
       </c>
       <c r="C461" s="8" t="inlineStr">
         <is>
-          <t>W2G01B19  m  800.0
-Montare cablu U1KV gr 1,301-1,500 Kg/M cu sau al sant pat nisip cu obstac cu tract manuala</t>
+          <t>$3275630  m  100.0
+CABLURI ELECTRICE CYABY-F 3X95+50 , 71760471360100 ICME ECAB</t>
         </is>
       </c>
       <c r="D461" s="9" t="inlineStr">
@@ -9902,31 +9903,31 @@
         </is>
       </c>
     </row>
-    <row r="462" ht="40" customHeight="1">
-      <c r="A462" s="7" t="n">
+    <row r="462" ht="20" customHeight="1">
+      <c r="A462" s="6" t="inlineStr">
+        <is>
+          <t>Categoria de lucrari: CANALIZARE</t>
+        </is>
+      </c>
+    </row>
+    <row r="463" ht="40" customHeight="1">
+      <c r="A463" s="7" t="n">
         <v>422</v>
       </c>
-      <c r="B462" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C462" s="8" t="inlineStr">
-        <is>
-          <t>W2A16A1  buc  38.0
-Stalp simplu teava otel in fundatie turnata teren N0rmal</t>
-        </is>
-      </c>
-      <c r="D462" s="9" t="inlineStr">
-        <is>
-          <t>ARTICOL SUPLIMENTAR ÎN OFERTĂ</t>
-        </is>
-      </c>
-    </row>
-    <row r="463" ht="20" customHeight="1">
-      <c r="A463" s="6" t="inlineStr">
-        <is>
-          <t>Categoria de lucrari: TELECOMUNICATII</t>
+      <c r="B463" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C463" s="8" t="inlineStr">
+        <is>
+          <t>TRI1AA01C2  tona  64.98
+Incarcarea materialelor, grupa a-grele si marunte,prin aruncare rampa sau teren-auto categ.2</t>
+        </is>
+      </c>
+      <c r="D463" s="9" t="inlineStr">
+        <is>
+          <t>ARTICOL SUPLIMENTAR ÎN OFERTĂ</t>
         </is>
       </c>
     </row>
@@ -9941,8 +9942,8 @@
       </c>
       <c r="C464" s="8" t="inlineStr">
         <is>
-          <t>$67185061  m  200.0
-BANDA AVERTIZOARE PVC INSCRIPTIONATA PENTRU CABLU TELECOMUNICATII ÎN SAPATURA 1 MM GROSIME</t>
+          <t>IA37E1  buc  2.0
+Rezervor depozit pentru combustibil lichid,cilindric capacitate 30000 L.</t>
         </is>
       </c>
       <c r="D464" s="9" t="inlineStr">
@@ -9951,52 +9952,51 @@
         </is>
       </c>
     </row>
-    <row r="465" ht="40" customHeight="1">
-      <c r="A465" s="7" t="n">
-        <v>424</v>
-      </c>
-      <c r="B465" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C465" s="8" t="inlineStr">
-        <is>
-          <t>W2H04A1  mc  16.0
-Strat nisip asezat in sant pentru protejarea cablurilor la lucr in prof netipizat material: manopera: utilaj: transport:</t>
-        </is>
-      </c>
-      <c r="D465" s="9" t="inlineStr">
-        <is>
-          <t>ARTICOL SUPLIMENTAR ÎN OFERTĂ</t>
+    <row r="465" ht="20" customHeight="1">
+      <c r="A465" s="6" t="inlineStr">
+        <is>
+          <t>Categoria de lucrari: MONTAJ SISTEM PANOU FOTOVOLTAICE</t>
         </is>
       </c>
     </row>
     <row r="466" ht="40" customHeight="1">
       <c r="A466" s="7" t="n">
+        <v>424</v>
+      </c>
+      <c r="B466" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C466" s="8" t="inlineStr">
+        <is>
+          <t>W1C01A1  buc  1.0
+ASIMILAT - MONTARE PANOURI FOTOVOLTAICE</t>
+        </is>
+      </c>
+      <c r="D466" s="9" t="inlineStr">
+        <is>
+          <t>ARTICOL SUPLIMENTAR ÎN OFERTĂ</t>
+        </is>
+      </c>
+    </row>
+    <row r="467" ht="40" customHeight="1">
+      <c r="A467" s="7" t="n">
         <v>425</v>
       </c>
-      <c r="B466" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C466" s="8" t="inlineStr">
-        <is>
-          <t>TRI1AA01C2  tona  8.42
-Incarcarea materialelor, grupa a-grele si marunte, prin aruncare rampa sau teren-auto categ.2</t>
-        </is>
-      </c>
-      <c r="D466" s="9" t="inlineStr">
-        <is>
-          <t>ARTICOL SUPLIMENTAR ÎN OFERTĂ</t>
-        </is>
-      </c>
-    </row>
-    <row r="467" ht="20" customHeight="1">
-      <c r="A467" s="6" t="inlineStr">
-        <is>
-          <t>Categoria de lucrari: SISTEM SUPRAVEGHEREA VIDEO -OB2</t>
+      <c r="B467" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C467" s="8" t="inlineStr">
+        <is>
+          <t>S7064  kg  45.0</t>
+        </is>
+      </c>
+      <c r="D467" s="9" t="inlineStr">
+        <is>
+          <t>ARTICOL SUPLIMENTAR ÎN OFERTĂ</t>
         </is>
       </c>
     </row>
@@ -10011,8 +10011,8 @@
       </c>
       <c r="C468" s="8" t="inlineStr">
         <is>
-          <t>$226288    0.0
-SISTEM SUPRAVEGHEREA VIDEO -OB2 e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
+          <t>$32745841  kg  1979.25
+OTEL BETON BST500 6-8 mm (BARA) 12 M</t>
         </is>
       </c>
       <c r="D468" s="9" t="inlineStr">
@@ -10021,31 +10021,31 @@
         </is>
       </c>
     </row>
-    <row r="469" ht="20" customHeight="1">
-      <c r="A469" s="6" t="inlineStr">
-        <is>
-          <t>Categoria de lucrari: INSTALATII VENTILATIE OB. 4</t>
-        </is>
-      </c>
-    </row>
-    <row r="470" ht="40" customHeight="1">
-      <c r="A470" s="7" t="n">
+    <row r="469" ht="40" customHeight="1">
+      <c r="A469" s="7" t="n">
         <v>427</v>
       </c>
-      <c r="B470" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C470" s="8" t="inlineStr">
-        <is>
-          <t>$1401  buc  2.0
-2500 MM montata pe canal material: manopera: utilaj: transport:</t>
-        </is>
-      </c>
-      <c r="D470" s="9" t="inlineStr">
-        <is>
-          <t>ARTICOL SUPLIMENTAR ÎN OFERTĂ</t>
+      <c r="B469" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C469" s="8" t="inlineStr">
+        <is>
+          <t>$32745861  kg  2324.35
+OTEL BETON BST500 10-12 mm (BARA) 12 M</t>
+        </is>
+      </c>
+      <c r="D469" s="9" t="inlineStr">
+        <is>
+          <t>ARTICOL SUPLIMENTAR ÎN OFERTĂ</t>
+        </is>
+      </c>
+    </row>
+    <row r="470" ht="20" customHeight="1">
+      <c r="A470" s="6" t="inlineStr">
+        <is>
+          <t>Categoria de lucrari: INSTAI.ATII VENTILATIE OB.2 eDevize e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar (fara TVA) - Lei - TOTALUL (fara TVA) - Lei - 0 1 2 3 4 5 = 3 x 4 1 VC01C1 - Montarea ventilatorului axial GR. totala 50- 200Kg buc 4.000 325.09 1,300.38 material: 102.34 409.38 manopera: 222.75 891.00 utilaj: 0.00 0.00 transport: 0.00 0.00 1 3270546 - VENTILATOR BAIE D=100MM, MODEL "EOL 100T" TIMER buc 4.000 178.00 712.00 2 VB14D1 - Priza de aer det tip 61/105 avind perimetrul 1401-2500 MM montata pe canal buc 4.000 71.47 285.90 material: 32.78 131.10 manopera: 38.70 154.80 utilaj: 0.00 0.00 transport: 0.00 0.00 2 7002221 - GRILA VENTILATIE DN110 MM BUC 4.000 135.00 540.00 3 VB30A1 - Anemostat plan patrat det tip 61/272 buc 4.000 69.78 279.14 material: 6.78 27.14 manopera: 63.00 252.00 utilaj: 0.00 0.00 transport: 0.00 0.00 3 2997173 - GRILA TRANSFER CU IZOLARE FONICA, ALUMINIU MONTAT IN USA 300X200 INCLUSIV CONTRARAMA buc 4.000 185.00 740.00 4 VA02B08 - Canale drepte confectionata pe sant cu perim sect de 400- 700 mm cu sect circ din tabla zinc de 0. 5 mm mp 5.000 165.79 828.96 material: 97.99 489.96 manopera: 67.80 339.00 utilaj: 0.00 0.00 transport: 0.00 0.00 4 7000777 - TUBUILATURA CIRCULARA RIGIDA D=100 NEIZOLATA, INCLUSIV PIESE SPECIALA SI SUPORTI SUPORT X m 15.000 35.00 525.00 5 VC23A1 - Confectionare dispoz. sust-ancor. pentru aparate canale piese spec. din otel prof. greut/buc sub 5 Kg. kg 10.000 26.70 266.99 material: 10.53 105.29 manopera: 16.17 161.69 utilaj: 0.00 0.00 transport: 0.00 0.00 Deviz "226248" - Formular F3 Formular generat cu programul @Devize (www.eDevize.ro) Pagina 1 din 2</t>
         </is>
       </c>
     </row>
@@ -10060,8 +10060,8 @@
       </c>
       <c r="C471" s="8" t="inlineStr">
         <is>
-          <t>$226538    0.0
-INSTALATII VENTILATIE OB 5 e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
+          <t>$1401  buc  4.0
+2500 MM montata pe canal material: manopera: utilaj: transport:</t>
         </is>
       </c>
       <c r="D471" s="9" t="inlineStr">
@@ -10070,136 +10070,136 @@
         </is>
       </c>
     </row>
-    <row r="472" ht="20" customHeight="1">
-      <c r="A472" s="6" t="inlineStr">
+    <row r="472" ht="40" customHeight="1">
+      <c r="A472" s="7" t="n">
+        <v>429</v>
+      </c>
+      <c r="B472" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C472" s="8" t="inlineStr">
+        <is>
+          <t>$226248    0.0
+INSTAI.ATII VENTILATIE OB.2 eDevize e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
+        </is>
+      </c>
+      <c r="D472" s="9" t="inlineStr">
+        <is>
+          <t>ARTICOL SUPLIMENTAR ÎN OFERTĂ</t>
+        </is>
+      </c>
+    </row>
+    <row r="473" ht="20" customHeight="1">
+      <c r="A473" s="6" t="inlineStr">
+        <is>
+          <t>Categoria de lucrari: ALIMENTARE CU APA</t>
+        </is>
+      </c>
+    </row>
+    <row r="474" ht="40" customHeight="1">
+      <c r="A474" s="7" t="n">
+        <v>430</v>
+      </c>
+      <c r="B474" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C474" s="8" t="inlineStr">
+        <is>
+          <t>TRI1AA01C2  tona  117.8
+Incarcarea materialelor, grupa a-grele si marunte,prin aruncare rampa sau teren-auto categ.2</t>
+        </is>
+      </c>
+      <c r="D474" s="9" t="inlineStr">
+        <is>
+          <t>ARTICOL SUPLIMENTAR ÎN OFERTĂ</t>
+        </is>
+      </c>
+    </row>
+    <row r="475" ht="40" customHeight="1">
+      <c r="A475" s="7" t="n">
+        <v>431</v>
+      </c>
+      <c r="B475" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C475" s="8" t="inlineStr">
+        <is>
+          <t>$6716997  m  345.0
+BANDA PVC CU INSERTIE DE METAL DETECTABIL</t>
+        </is>
+      </c>
+      <c r="D475" s="9" t="inlineStr">
+        <is>
+          <t>ARTICOL SUPLIMENTAR ÎN OFERTĂ</t>
+        </is>
+      </c>
+    </row>
+    <row r="476" ht="20" customHeight="1">
+      <c r="A476" s="6" t="inlineStr">
         <is>
           <t>Categoria de lucrari: CHELTUIELI CONEXE ORGANIZARII DE SANTIER</t>
         </is>
       </c>
     </row>
-    <row r="473" ht="40" customHeight="1">
-      <c r="A473" s="7" t="n">
-        <v>429</v>
-      </c>
-      <c r="B473" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C473" s="8" t="inlineStr">
+    <row r="477" ht="40" customHeight="1">
+      <c r="A477" s="7" t="n">
+        <v>432</v>
+      </c>
+      <c r="B477" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C477" s="8" t="inlineStr">
         <is>
           <t>CHELT  lei  30000.0
 CHELTUIELI CONEXE ORGANIZARE SANTIER</t>
         </is>
       </c>
-      <c r="D473" s="9" t="inlineStr">
-        <is>
-          <t>ARTICOL SUPLIMENTAR ÎN OFERTĂ</t>
-        </is>
-      </c>
-    </row>
-    <row r="474" ht="20" customHeight="1">
-      <c r="A474" s="6" t="inlineStr">
+      <c r="D477" s="9" t="inlineStr">
+        <is>
+          <t>ARTICOL SUPLIMENTAR ÎN OFERTĂ</t>
+        </is>
+      </c>
+    </row>
+    <row r="478" ht="20" customHeight="1">
+      <c r="A478" s="6" t="inlineStr">
+        <is>
+          <t>Categoria de lucrari: SISTEM SUPRAVEGHEREA VIDEO -OB2</t>
+        </is>
+      </c>
+    </row>
+    <row r="479" ht="40" customHeight="1">
+      <c r="A479" s="7" t="n">
+        <v>433</v>
+      </c>
+      <c r="B479" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C479" s="8" t="inlineStr">
+        <is>
+          <t>$226288    0.0
+SISTEM SUPRAVEGHEREA VIDEO -OB2 e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
+        </is>
+      </c>
+      <c r="D479" s="9" t="inlineStr">
+        <is>
+          <t>ARTICOL SUPLIMENTAR ÎN OFERTĂ</t>
+        </is>
+      </c>
+    </row>
+    <row r="480" ht="20" customHeight="1">
+      <c r="A480" s="6" t="inlineStr">
         <is>
           <t>Categoria de lucrari: SPATII VERZI e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar (fara TVA) - Lei - TOTALUL (fara TVA) - Lei - 0 1 2 3 4 5 = 3 x 4 1 TSH01A1 - Degajarea terenului de corpuri straine de corpuri straine 100 mp 59.180 212.10 12,552.08 material: 0.00 0.00 manopera: 212.10 12,552.08 utilaj: 0.00 0.00 transport: 0.00 0.00 2 TSC02C11 - Sapatura mecanica cu excavator pe pneuri de 0.12-0.39 mc,cu comanda hidraulica, in : pamant cu umiditate naturala descarcare auto in teren catg 1 in conditiile gospodaririi apelor 100 mc 17.750 447.45 7,942.24 material: 0.00 0.00 manopera: 0.00 0.00 utilaj: 447.45 7,942.24 transport: 0.00 0.00 3 TRA01A10P - Transportul rutier al pamintului sau molozului cu autobasculanta dist .= 10 km $ tona 3,373.370 2.00 6,747.75 material: 0.00 0.00 manopera: 0.00 1.01 utilaj: 0.00 0.00 transport: 2.00 6,746.74 4 TSE04A1 - Nivelarea terenului natural si platformelor de terasamente cu buldozer pe tractor pe senile, prin taierea damburilor si impingerea in goluri a pamantului sapat,cu: buldozer pe tractor pe senile de 65-80 CP teren catg. 1 si 2 100 mp 59.180 12.50 739.75 material: 0.00 0.00 manopera: 0.00 0.00 utilaj: 12.50 739.75 transport: 0.00 0.00 5 TSE01A1 - Nivelarea manuala a terenurilor si platformelor,cu denivelari de 10-20 CM,in: teren usor 100 mp 59.180 177.00 10,474.86 material: 0.00 0.00 manopera: 177.00 10,474.86 utilaj: 0.00 0.00 transport: 0.00 0.00 6 TSH05D1 - Asternerea uniforma a stratului de pamant vegetal,pe teren orizontal sau cu panta la 20 %,cu pastrarea structurii, in straturi de : 30 cm grosime mp 5,918.000 5.40 31,957.20 material: 0.00 0.00 manopera: 5.40 31,957.20 utilaj: 0.00 0.00 transport: 0.00 0.00 6 2100001 - Pamant vegetal mc 1,775.000 230.00 408,250.00 Deviz "226348" - Formular F3 Formular generat cu programul @Devize (www.eDevize.ro) Pagina 1 din 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="475" ht="40" customHeight="1">
-      <c r="A475" s="7" t="n">
-        <v>430</v>
-      </c>
-      <c r="B475" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C475" s="8" t="inlineStr">
-        <is>
-          <t>$226348    0.0
-SPATII VERZI e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
-        </is>
-      </c>
-      <c r="D475" s="9" t="inlineStr">
-        <is>
-          <t>ARTICOL SUPLIMENTAR ÎN OFERTĂ</t>
-        </is>
-      </c>
-    </row>
-    <row r="476" ht="20" customHeight="1">
-      <c r="A476" s="6" t="inlineStr">
-        <is>
-          <t>Categoria de lucrari: CANALIZARE</t>
-        </is>
-      </c>
-    </row>
-    <row r="477" ht="40" customHeight="1">
-      <c r="A477" s="7" t="n">
-        <v>431</v>
-      </c>
-      <c r="B477" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C477" s="8" t="inlineStr">
-        <is>
-          <t>TRI1AA01C2  tona  64.98
-Incarcarea materialelor, grupa a-grele si marunte,prin aruncare rampa sau teren-auto categ.2</t>
-        </is>
-      </c>
-      <c r="D477" s="9" t="inlineStr">
-        <is>
-          <t>ARTICOL SUPLIMENTAR ÎN OFERTĂ</t>
-        </is>
-      </c>
-    </row>
-    <row r="478" ht="40" customHeight="1">
-      <c r="A478" s="7" t="n">
-        <v>432</v>
-      </c>
-      <c r="B478" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C478" s="8" t="inlineStr">
-        <is>
-          <t>IA37E1  buc  2.0
-Rezervor depozit pentru combustibil lichid,cilindric capacitate 30000 L.</t>
-        </is>
-      </c>
-      <c r="D478" s="9" t="inlineStr">
-        <is>
-          <t>ARTICOL SUPLIMENTAR ÎN OFERTĂ</t>
-        </is>
-      </c>
-    </row>
-    <row r="479" ht="20" customHeight="1">
-      <c r="A479" s="6" t="inlineStr">
-        <is>
-          <t>Categoria de lucrari: INSTALATIE VENTILATIE OB 4 e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar (fara TVA) - Lei - TOTALUL (fara TVA) - Lei - 0 1 2 3 4 5 = 3 x 4 1 VC01C1 - Montarea ventilatorului axial GR. totala 50- 200Kg buc 4.000 325.09 1,300.38 material: 102.34 409.38 manopera: 222.75 891.00 utilaj: 0.00 0.00 transport: 0.00 0.00 1 3270546 - VENTILATOR BAIE D=100MM, MODEL "EOL 100T" TIMER buc 3.000 178.00 534.00 1 3272502 - VENTILATOR BAIE SILENT-100CZ-D=100-230V- 95MC/H-SOLER PALAU buc 1.000 225.00 225.00 2 VB14D1 - Priza de aer det tip 61/105 avind perimetrul 1401-2500 MM montata pe canal buc 1.000 71.47 71.47 material: 32.78 32.78 manopera: 38.70 38.70 utilaj: 0.00 0.00 transport: 0.00 0.00 2 7002221 - GRILA VENTILATIE DN110 MM BUC 1.000 135.00 135.00 3 VB14D1 - Priza de aer det tip 61/105 avind perimetrul 1401-2500 MM montata pe canal buc 2.000 71.47 142.95 material: 32.78 65.55 manopera: 38.70 77.40 utilaj: 0.00 0.00 transport: 0.00 0.00 3 2997228 - GRILA EXTERIOARA CU JALUZELE FIXE Dn125 cu jaluzele anti ploaie si plasa antiinsecte buc 2.000 35.00 70.00 4 VB30A1 - Anemostat plan patrat det tip 61/272 buc 4.000 69.78 279.14 material: 6.78 27.14 manopera: 63.00 252.00 utilaj: 0.00 0.00 transport: 0.00 0.00 4 2997173 - GRILA TRANSFER CU IZOLARE FONICA, ALUMINIU MONTAT IN USA 300X200 INCLUSIV CONTRARAMA buc 4.000 185.00 740.00 5 VA02B08 - Canale drepte confectionata pe sant cu perim sect de 400- 700 mm cu sect circ din tabla zinc de 0. 5 mm mp 4.500 165.79 746.07 material: 97.99 440.97 manopera: 67.80 305.10 utilaj: 0.00 0.00 transport: 0.00 0.00 Deviz "226448" - Formular F3 Formular generat cu programul @Devize (www.eDevize.ro) Pagina 1 din 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="480" ht="40" customHeight="1">
-      <c r="A480" s="7" t="n">
-        <v>433</v>
-      </c>
-      <c r="B480" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C480" s="8" t="inlineStr">
-        <is>
-          <t>$226448    0.0
-INSTALATIE VENTILATIE OB 4 e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
-        </is>
-      </c>
-      <c r="D480" s="9" t="inlineStr">
-        <is>
-          <t>ARTICOL SUPLIMENTAR ÎN OFERTĂ</t>
         </is>
       </c>
     </row>
@@ -10214,8 +10214,8 @@
       </c>
       <c r="C481" s="8" t="inlineStr">
         <is>
-          <t>$1401  buc  2.0
-2500 MM montata pe canal material: manopera: utilaj: transport:</t>
+          <t>$226348    0.0
+SPATII VERZI e Devize Formular F3 Lista cu cantitati de lucrari pe categorii de lucrari SECTIUNEA TEHNICA SECTIUNEA FINANCIARA Nr. Capitol de lucrari U.M. Cantitatea Pretul unitar - Lei - TOTALUL - Lei -</t>
         </is>
       </c>
       <c r="D481" s="9" t="inlineStr">
@@ -10227,9 +10227,9 @@
   </sheetData>
   <mergeCells count="41">
     <mergeCell ref="A414:D414"/>
-    <mergeCell ref="A479:D479"/>
     <mergeCell ref="A424:D424"/>
     <mergeCell ref="A439:D439"/>
+    <mergeCell ref="A470:D470"/>
     <mergeCell ref="A395:D395"/>
     <mergeCell ref="A411:D411"/>
     <mergeCell ref="A324:D324"/>
@@ -10239,33 +10239,33 @@
     <mergeCell ref="A152:D152"/>
     <mergeCell ref="A190:D190"/>
     <mergeCell ref="A445:D445"/>
-    <mergeCell ref="A450:D450"/>
     <mergeCell ref="A28:D28"/>
     <mergeCell ref="A391:D391"/>
     <mergeCell ref="A173:D173"/>
     <mergeCell ref="A245:D245"/>
     <mergeCell ref="A83:D83"/>
+    <mergeCell ref="A480:D480"/>
     <mergeCell ref="A157:D157"/>
     <mergeCell ref="A403:D403"/>
     <mergeCell ref="A437:D437"/>
     <mergeCell ref="A431:D431"/>
     <mergeCell ref="A387:D387"/>
+    <mergeCell ref="A462:D462"/>
     <mergeCell ref="A476:D476"/>
     <mergeCell ref="A296:D296"/>
-    <mergeCell ref="A467:D467"/>
     <mergeCell ref="A281:D281"/>
     <mergeCell ref="A119:D119"/>
+    <mergeCell ref="A473:D473"/>
     <mergeCell ref="A442:D442"/>
+    <mergeCell ref="A478:D478"/>
     <mergeCell ref="A7:D7"/>
-    <mergeCell ref="A463:D463"/>
     <mergeCell ref="A363:D363"/>
-    <mergeCell ref="A472:D472"/>
-    <mergeCell ref="A469:D469"/>
+    <mergeCell ref="A465:D465"/>
     <mergeCell ref="A434:D434"/>
     <mergeCell ref="A428:D428"/>
-    <mergeCell ref="A474:D474"/>
     <mergeCell ref="A179:D179"/>
     <mergeCell ref="A213:D213"/>
+    <mergeCell ref="A449:D449"/>
     <mergeCell ref="A374:D374"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>